<commit_message>
📊 Update KOSPI Top200 operating profit - 2026-04-01
</commit_message>
<xml_diff>
--- a/top200_operating_profit_kospi.xlsx
+++ b/top200_operating_profit_kospi.xlsx
@@ -769,20 +769,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>95251.38</v>
+        <v>175694.57</v>
       </c>
       <c r="D13" t="n">
-        <v>20226.04</v>
+        <v>20427.26</v>
       </c>
       <c r="E13" t="n">
-        <v>14675.05</v>
+        <v>14224.81</v>
       </c>
       <c r="F13" t="n">
-        <v>246513.33</v>
+        <v>261990.62</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -796,20 +796,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>70193.3</v>
+        <v>95251.38</v>
       </c>
       <c r="D14" t="n">
-        <v>19455.32</v>
+        <v>20226.04</v>
       </c>
       <c r="E14" t="n">
-        <v>18829.69</v>
+        <v>14675.05</v>
       </c>
       <c r="F14" t="n">
-        <v>203411.99</v>
+        <v>246513.33</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -823,20 +823,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>NAVER</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>25565.03</v>
+        <v>70193.3</v>
       </c>
       <c r="D15" t="n">
-        <v>18008.63</v>
+        <v>19455.32</v>
       </c>
       <c r="E15" t="n">
-        <v>16198.67</v>
+        <v>18829.69</v>
       </c>
       <c r="F15" t="n">
-        <v>376723.03</v>
+        <v>203411.99</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -850,20 +850,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>한국가스공사</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>340184.34</v>
+        <v>25565.03</v>
       </c>
       <c r="D16" t="n">
-        <v>17919.34</v>
+        <v>18008.63</v>
       </c>
       <c r="E16" t="n">
-        <v>6992.64</v>
+        <v>16198.67</v>
       </c>
       <c r="F16" t="n">
-        <v>500856.22</v>
+        <v>376723.03</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -877,20 +877,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>한국가스공사</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20386.69</v>
+        <v>340184.34</v>
       </c>
       <c r="D17" t="n">
-        <v>17583.21</v>
+        <v>17919.34</v>
       </c>
       <c r="E17" t="n">
-        <v>17455.71</v>
+        <v>6992.64</v>
       </c>
       <c r="F17" t="n">
-        <v>266693.48</v>
+        <v>500856.22</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -904,20 +904,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>현대모비스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>362568.23</v>
+        <v>20386.69</v>
       </c>
       <c r="D18" t="n">
-        <v>17369.59</v>
+        <v>17583.21</v>
       </c>
       <c r="E18" t="n">
-        <v>21124.41</v>
+        <v>17455.71</v>
       </c>
       <c r="F18" t="n">
-        <v>385370</v>
+        <v>266693.48</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -931,20 +931,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>현대모비스</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>306864.48</v>
+        <v>362568.23</v>
       </c>
       <c r="D19" t="n">
-        <v>16664.61</v>
+        <v>17369.59</v>
       </c>
       <c r="E19" t="n">
-        <v>16997.62</v>
+        <v>21124.41</v>
       </c>
       <c r="F19" t="n">
-        <v>3099482.94</v>
+        <v>385370</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -958,20 +958,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>165018.52</v>
+        <v>306864.48</v>
       </c>
       <c r="D20" t="n">
-        <v>15392.52</v>
+        <v>16664.61</v>
       </c>
       <c r="E20" t="n">
-        <v>9649.299999999999</v>
+        <v>16997.62</v>
       </c>
       <c r="F20" t="n">
-        <v>384566.48</v>
+        <v>3099482.94</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -985,20 +985,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>107211.77</v>
+        <v>225317.96</v>
       </c>
       <c r="D21" t="n">
-        <v>14232</v>
+        <v>15612.98</v>
       </c>
       <c r="E21" t="n">
-        <v>18512.82</v>
+        <v>14605.15</v>
       </c>
       <c r="F21" t="n">
-        <v>329632.63</v>
+        <v>152215.75</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1012,20 +1012,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>현대해상</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>172193.14</v>
+        <v>165018.52</v>
       </c>
       <c r="D22" t="n">
-        <v>14018.71</v>
+        <v>15392.52</v>
       </c>
       <c r="E22" t="n">
-        <v>10306.84</v>
+        <v>9649.299999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>479776.79</v>
+        <v>384566.48</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1039,20 +1039,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>193240.24</v>
+        <v>107211.77</v>
       </c>
       <c r="D23" t="n">
-        <v>13049.73</v>
+        <v>14232</v>
       </c>
       <c r="E23" t="n">
-        <v>10617.53</v>
+        <v>18512.82</v>
       </c>
       <c r="F23" t="n">
-        <v>296775.87</v>
+        <v>329632.63</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1066,20 +1066,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>현대해상</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>216347.35</v>
+        <v>172193.14</v>
       </c>
       <c r="D24" t="n">
-        <v>12477.07</v>
+        <v>14018.71</v>
       </c>
       <c r="E24" t="n">
-        <v>11249.46</v>
+        <v>10306.84</v>
       </c>
       <c r="F24" t="n">
-        <v>138411.21</v>
+        <v>479776.79</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1093,20 +1093,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>키움증권</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>13584.64</v>
+        <v>157151.87</v>
       </c>
       <c r="D25" t="n">
-        <v>12203.67</v>
+        <v>13254.58</v>
       </c>
       <c r="E25" t="n">
-        <v>12276.08</v>
+        <v>10994.04</v>
       </c>
       <c r="F25" t="n">
-        <v>52404.74</v>
+        <v>688072.48</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1120,20 +1120,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>고려아연</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>105342.41</v>
+        <v>193240.24</v>
       </c>
       <c r="D26" t="n">
-        <v>11795.5</v>
+        <v>13049.73</v>
       </c>
       <c r="E26" t="n">
-        <v>7715.72</v>
+        <v>10617.53</v>
       </c>
       <c r="F26" t="n">
-        <v>169216.42</v>
+        <v>296775.87</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1147,20 +1147,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>메리츠금융지주</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>129035.94</v>
+        <v>13584.64</v>
       </c>
       <c r="D27" t="n">
-        <v>11540.03</v>
+        <v>12203.67</v>
       </c>
       <c r="E27" t="n">
-        <v>13441.99</v>
+        <v>12276.08</v>
       </c>
       <c r="F27" t="n">
-        <v>197246.46</v>
+        <v>52404.74</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1174,20 +1174,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>고려아연</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>12625.33</v>
+        <v>105342.41</v>
       </c>
       <c r="D28" t="n">
-        <v>11233.01</v>
+        <v>11795.5</v>
       </c>
       <c r="E28" t="n">
-        <v>11233.32</v>
+        <v>7715.72</v>
       </c>
       <c r="F28" t="n">
-        <v>263530.37</v>
+        <v>169216.42</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1201,20 +1201,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>129366.6</v>
+        <v>129035.94</v>
       </c>
       <c r="D29" t="n">
-        <v>11054.9</v>
+        <v>11540.03</v>
       </c>
       <c r="E29" t="n">
-        <v>8188.16</v>
+        <v>13441.99</v>
       </c>
       <c r="F29" t="n">
-        <v>569763.86</v>
+        <v>197246.46</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1228,20 +1228,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>크래프톤</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28856.5</v>
+        <v>12625.33</v>
       </c>
       <c r="D30" t="n">
-        <v>10627.18</v>
+        <v>11233.01</v>
       </c>
       <c r="E30" t="n">
-        <v>7351.51</v>
+        <v>11233.32</v>
       </c>
       <c r="F30" t="n">
-        <v>81595.94</v>
+        <v>263530.37</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1255,20 +1255,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>키움증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>102101.84</v>
+        <v>129366.6</v>
       </c>
       <c r="D31" t="n">
-        <v>10247.33</v>
+        <v>11054.9</v>
       </c>
       <c r="E31" t="n">
-        <v>8150.78</v>
+        <v>8188.16</v>
       </c>
       <c r="F31" t="n">
-        <v>456778.63</v>
+        <v>569763.86</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1282,20 +1282,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>크래프톤</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>41454.75</v>
+        <v>28856.5</v>
       </c>
       <c r="D32" t="n">
-        <v>10007.17</v>
+        <v>10627.18</v>
       </c>
       <c r="E32" t="n">
-        <v>9198.23</v>
+        <v>7351.51</v>
       </c>
       <c r="F32" t="n">
-        <v>113642.92</v>
+        <v>81595.94</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1309,20 +1309,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>KT&amp;G</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>56949.95</v>
+        <v>41454.75</v>
       </c>
       <c r="D33" t="n">
-        <v>9988.799999999999</v>
+        <v>10007.17</v>
       </c>
       <c r="E33" t="n">
-        <v>7433.49</v>
+        <v>9198.23</v>
       </c>
       <c r="F33" t="n">
-        <v>90510.12</v>
+        <v>113642.92</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1336,20 +1336,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>14033.1</v>
+        <v>56949.95</v>
       </c>
       <c r="D34" t="n">
-        <v>9768.25</v>
+        <v>9988.799999999999</v>
       </c>
       <c r="E34" t="n">
-        <v>4948.78</v>
+        <v>7433.49</v>
       </c>
       <c r="F34" t="n">
-        <v>518155.85</v>
+        <v>90510.12</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1363,20 +1363,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>165863.46</v>
+        <v>14033.1</v>
       </c>
       <c r="D35" t="n">
-        <v>9241.860000000001</v>
+        <v>9768.25</v>
       </c>
       <c r="E35" t="n">
-        <v>6991.3</v>
+        <v>4948.78</v>
       </c>
       <c r="F35" t="n">
-        <v>951663.41</v>
+        <v>518155.85</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1390,20 +1390,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>29286.38</v>
+        <v>165863.46</v>
       </c>
       <c r="D36" t="n">
-        <v>9189.52</v>
+        <v>9241.860000000001</v>
       </c>
       <c r="E36" t="n">
-        <v>8475.43</v>
+        <v>6991.3</v>
       </c>
       <c r="F36" t="n">
-        <v>218130.1</v>
+        <v>951663.41</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1417,20 +1417,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>142042.31</v>
+        <v>29286.38</v>
       </c>
       <c r="D37" t="n">
-        <v>9117.41</v>
+        <v>9189.52</v>
       </c>
       <c r="E37" t="n">
-        <v>5427.99</v>
+        <v>8475.43</v>
       </c>
       <c r="F37" t="n">
-        <v>187145.25</v>
+        <v>218130.1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1444,20 +1444,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>33811.39</v>
+        <v>142042.31</v>
       </c>
       <c r="D38" t="n">
-        <v>8891.57</v>
+        <v>9117.41</v>
       </c>
       <c r="E38" t="n">
-        <v>6364.38</v>
+        <v>5427.99</v>
       </c>
       <c r="F38" t="n">
-        <v>35038.24</v>
+        <v>187145.25</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1471,20 +1471,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>HD현대일렉트릭</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>94508.34</v>
+        <v>33811.39</v>
       </c>
       <c r="D39" t="n">
-        <v>8791.6</v>
+        <v>8891.57</v>
       </c>
       <c r="E39" t="n">
-        <v>6259.15</v>
+        <v>6364.38</v>
       </c>
       <c r="F39" t="n">
-        <v>592814.76</v>
+        <v>35038.24</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1498,20 +1498,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>106349.53</v>
+        <v>94508.34</v>
       </c>
       <c r="D40" t="n">
-        <v>8670.6</v>
+        <v>8791.6</v>
       </c>
       <c r="E40" t="n">
-        <v>5403.24</v>
+        <v>6259.15</v>
       </c>
       <c r="F40" t="n">
-        <v>147746.88</v>
+        <v>592814.76</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1525,20 +1525,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>포스코인터내셔널</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>269565.98</v>
+        <v>106349.53</v>
       </c>
       <c r="D41" t="n">
-        <v>8546.379999999999</v>
+        <v>8670.6</v>
       </c>
       <c r="E41" t="n">
-        <v>5138.3</v>
+        <v>5403.24</v>
       </c>
       <c r="F41" t="n">
-        <v>137253.92</v>
+        <v>147746.88</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1552,20 +1552,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>삼성카드</t>
+          <t>포스코인터내셔널</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>41901.45</v>
+        <v>269565.98</v>
       </c>
       <c r="D42" t="n">
-        <v>8526.040000000001</v>
+        <v>8546.379999999999</v>
       </c>
       <c r="E42" t="n">
-        <v>6438.03</v>
+        <v>5138.3</v>
       </c>
       <c r="F42" t="n">
-        <v>314635.2</v>
+        <v>137253.92</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1579,20 +1579,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>삼성카드</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>36122.94</v>
+        <v>41901.45</v>
       </c>
       <c r="D43" t="n">
-        <v>8131.63</v>
+        <v>8526.040000000001</v>
       </c>
       <c r="E43" t="n">
-        <v>13440.8</v>
+        <v>6438.03</v>
       </c>
       <c r="F43" t="n">
-        <v>263989.93</v>
+        <v>314635.2</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1606,20 +1606,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>120510.68</v>
+        <v>36122.94</v>
       </c>
       <c r="D44" t="n">
-        <v>8118.42</v>
+        <v>8131.63</v>
       </c>
       <c r="E44" t="n">
-        <v>4107.95</v>
+        <v>13440.8</v>
       </c>
       <c r="F44" t="n">
-        <v>251487.36</v>
+        <v>263989.93</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1633,20 +1633,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>144763.9</v>
+        <v>120510.68</v>
       </c>
       <c r="D45" t="n">
-        <v>7025.43</v>
+        <v>8118.42</v>
       </c>
       <c r="E45" t="n">
-        <v>6183.35</v>
+        <v>4107.95</v>
       </c>
       <c r="F45" t="n">
-        <v>194012.94</v>
+        <v>251487.36</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1660,20 +1660,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>7806.06</v>
+        <v>14937.54</v>
       </c>
       <c r="D46" t="n">
-        <v>6207.13</v>
+        <v>7006.49</v>
       </c>
       <c r="E46" t="n">
-        <v>6168.82</v>
+        <v>6143.35</v>
       </c>
       <c r="F46" t="n">
-        <v>109040.74</v>
+        <v>129011.26</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1687,20 +1687,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>카카오뱅크</t>
+          <t>한국금융지주</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>29456.21</v>
+        <v>7806.06</v>
       </c>
       <c r="D47" t="n">
-        <v>6068.8</v>
+        <v>6207.13</v>
       </c>
       <c r="E47" t="n">
-        <v>4400.65</v>
+        <v>6168.82</v>
       </c>
       <c r="F47" t="n">
-        <v>628052.8199999999</v>
+        <v>109040.74</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1714,20 +1714,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>코웨이</t>
+          <t>카카오뱅크</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>34685.41</v>
+        <v>29456.21</v>
       </c>
       <c r="D48" t="n">
-        <v>5958.42</v>
+        <v>6068.8</v>
       </c>
       <c r="E48" t="n">
-        <v>3990.59</v>
+        <v>4400.65</v>
       </c>
       <c r="F48" t="n">
-        <v>49158.47</v>
+        <v>628052.8199999999</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1741,20 +1741,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>LG</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6794.38</v>
+        <v>8849.889999999999</v>
       </c>
       <c r="D49" t="n">
-        <v>5904.66</v>
+        <v>5971.32</v>
       </c>
       <c r="E49" t="n">
-        <v>5616.36</v>
+        <v>8144.68</v>
       </c>
       <c r="F49" t="n">
-        <v>69810.25</v>
+        <v>103878.23</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -1768,20 +1768,20 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>코웨이</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>133221.44</v>
+        <v>34685.41</v>
       </c>
       <c r="D50" t="n">
-        <v>5824.59</v>
+        <v>5958.42</v>
       </c>
       <c r="E50" t="n">
-        <v>7205.7</v>
+        <v>3990.59</v>
       </c>
       <c r="F50" t="n">
-        <v>1221350.33</v>
+        <v>49158.47</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1795,20 +1795,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>삼성물산</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>212191.56</v>
+        <v>133221.44</v>
       </c>
       <c r="D51" t="n">
-        <v>5484.15</v>
+        <v>5824.59</v>
       </c>
       <c r="E51" t="n">
-        <v>10647.45</v>
+        <v>7205.7</v>
       </c>
       <c r="F51" t="n">
-        <v>639985.04</v>
+        <v>1221350.33</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1822,20 +1822,20 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>지역난방공사</t>
+          <t>삼성물산</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>39979.52</v>
+        <v>212191.56</v>
       </c>
       <c r="D52" t="n">
-        <v>5270.43</v>
+        <v>5484.15</v>
       </c>
       <c r="E52" t="n">
-        <v>3388.26</v>
+        <v>10647.45</v>
       </c>
       <c r="F52" t="n">
-        <v>82232.47</v>
+        <v>639985.04</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -1849,20 +1849,20 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>지역난방공사</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>54646.38</v>
+        <v>39979.52</v>
       </c>
       <c r="D53" t="n">
-        <v>5204.33</v>
+        <v>5270.43</v>
       </c>
       <c r="E53" t="n">
-        <v>4752.08</v>
+        <v>3388.26</v>
       </c>
       <c r="F53" t="n">
-        <v>84764.87</v>
+        <v>82232.47</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -1876,20 +1876,20 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>한화손해보험</t>
+          <t>삼성에스디에스</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>59675.46</v>
+        <v>54646.38</v>
       </c>
       <c r="D54" t="n">
-        <v>5033.89</v>
+        <v>5204.33</v>
       </c>
       <c r="E54" t="n">
-        <v>3822.76</v>
+        <v>4752.08</v>
       </c>
       <c r="F54" t="n">
-        <v>197526.8</v>
+        <v>84764.87</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -1903,20 +1903,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>한화손해보험</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>25951.01</v>
+        <v>59675.46</v>
       </c>
       <c r="D55" t="n">
-        <v>4919.7</v>
+        <v>5033.89</v>
       </c>
       <c r="E55" t="n">
-        <v>381.57</v>
+        <v>3822.76</v>
       </c>
       <c r="F55" t="n">
-        <v>116074.87</v>
+        <v>197526.8</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -1930,20 +1930,20 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>81002.07000000001</v>
+        <v>71170.23</v>
       </c>
       <c r="D56" t="n">
-        <v>4811.25</v>
+        <v>4960.06</v>
       </c>
       <c r="E56" t="n">
-        <v>399.67</v>
+        <v>5076.66</v>
       </c>
       <c r="F56" t="n">
-        <v>131632.9</v>
+        <v>148663.75</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -1961,16 +1961,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>40689.09</v>
+        <v>41440.72</v>
       </c>
       <c r="D57" t="n">
-        <v>4659.52</v>
+        <v>4850.72</v>
       </c>
       <c r="E57" t="n">
-        <v>2491.07</v>
+        <v>2983.47</v>
       </c>
       <c r="F57" t="n">
-        <v>101430.76</v>
+        <v>107163.79</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -1984,20 +1984,20 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>40978.14</v>
+        <v>81002.07000000001</v>
       </c>
       <c r="D58" t="n">
-        <v>4423.78</v>
+        <v>4811.25</v>
       </c>
       <c r="E58" t="n">
-        <v>2745.11</v>
+        <v>399.67</v>
       </c>
       <c r="F58" t="n">
-        <v>51014.56</v>
+        <v>131632.9</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2011,20 +2011,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>JB금융지주</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>5052.56</v>
+        <v>19018.34</v>
       </c>
       <c r="D59" t="n">
-        <v>4336.51</v>
+        <v>4713.97</v>
       </c>
       <c r="E59" t="n">
-        <v>4336.22</v>
+        <v>3553.03</v>
       </c>
       <c r="F59" t="n">
-        <v>34207.97</v>
+        <v>18927.11</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2038,20 +2038,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LG씨엔에스</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>54492.71</v>
+        <v>40978.14</v>
       </c>
       <c r="D60" t="n">
-        <v>4335.34</v>
+        <v>4423.78</v>
       </c>
       <c r="E60" t="n">
-        <v>3888.54</v>
+        <v>2745.11</v>
       </c>
       <c r="F60" t="n">
-        <v>48322.18</v>
+        <v>51014.56</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2065,20 +2065,20 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>S-Oil</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>361817.94</v>
+        <v>26808.61</v>
       </c>
       <c r="D61" t="n">
-        <v>4195.16</v>
+        <v>4402.42</v>
       </c>
       <c r="E61" t="n">
-        <v>-1967.06</v>
+        <v>2341.92</v>
       </c>
       <c r="F61" t="n">
-        <v>243693.17</v>
+        <v>115903.69</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2092,20 +2092,20 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>롯데쇼핑</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>81880.61</v>
+        <v>5260.74</v>
       </c>
       <c r="D62" t="n">
-        <v>4112.35</v>
+        <v>4391.82</v>
       </c>
       <c r="E62" t="n">
-        <v>1104.16</v>
+        <v>4020.47</v>
       </c>
       <c r="F62" t="n">
-        <v>303486.58</v>
+        <v>89930.52</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2119,20 +2119,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>F&amp;F</t>
+          <t>JB금융지주</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>15179.94</v>
+        <v>5052.56</v>
       </c>
       <c r="D63" t="n">
-        <v>4024.07</v>
+        <v>4336.51</v>
       </c>
       <c r="E63" t="n">
-        <v>3235.32</v>
+        <v>4336.22</v>
       </c>
       <c r="F63" t="n">
-        <v>19235.04</v>
+        <v>34207.97</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2146,20 +2146,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>LG씨엔에스</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>215960.08</v>
+        <v>54492.71</v>
       </c>
       <c r="D64" t="n">
-        <v>4007.06</v>
+        <v>4335.34</v>
       </c>
       <c r="E64" t="n">
-        <v>2592.17</v>
+        <v>3888.54</v>
       </c>
       <c r="F64" t="n">
-        <v>101904.14</v>
+        <v>48322.18</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2173,20 +2173,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>코리안리</t>
+          <t>롯데쇼핑</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>68031.78</v>
+        <v>81880.61</v>
       </c>
       <c r="D65" t="n">
-        <v>3994.96</v>
+        <v>4112.35</v>
       </c>
       <c r="E65" t="n">
-        <v>2858.73</v>
+        <v>1104.16</v>
       </c>
       <c r="F65" t="n">
-        <v>129267.22</v>
+        <v>303486.58</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2200,20 +2200,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>두산밥캣</t>
+          <t>금호타이어</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4903.43</v>
+        <v>35308.91</v>
       </c>
       <c r="D66" t="n">
-        <v>3935.42</v>
+        <v>4082.13</v>
       </c>
       <c r="E66" t="n">
-        <v>3690.68</v>
+        <v>3829.93</v>
       </c>
       <c r="F66" t="n">
-        <v>40606.56</v>
+        <v>39988.07</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2227,20 +2227,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>F&amp;F</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>63203.04</v>
+        <v>15179.94</v>
       </c>
       <c r="D67" t="n">
-        <v>3934.27</v>
+        <v>4024.07</v>
       </c>
       <c r="E67" t="n">
-        <v>-1703.05</v>
+        <v>3235.32</v>
       </c>
       <c r="F67" t="n">
-        <v>137568.74</v>
+        <v>19235.04</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2254,20 +2254,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>동양생명</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>34667.35</v>
+        <v>215960.08</v>
       </c>
       <c r="D68" t="n">
-        <v>3790.53</v>
+        <v>4007.06</v>
       </c>
       <c r="E68" t="n">
-        <v>3101.58</v>
+        <v>2592.17</v>
       </c>
       <c r="F68" t="n">
-        <v>345775.75</v>
+        <v>101904.14</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2281,20 +2281,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>코리안리</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>83779.08</v>
+        <v>68031.78</v>
       </c>
       <c r="D69" t="n">
-        <v>3559.4</v>
+        <v>3994.96</v>
       </c>
       <c r="E69" t="n">
-        <v>3918.63</v>
+        <v>2858.73</v>
       </c>
       <c r="F69" t="n">
-        <v>100939.74</v>
+        <v>129267.22</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2308,20 +2308,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CJ대한통운</t>
+          <t>두산밥캣</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>83538.53</v>
+        <v>4903.43</v>
       </c>
       <c r="D70" t="n">
-        <v>3531.28</v>
+        <v>3935.42</v>
       </c>
       <c r="E70" t="n">
-        <v>2069.36</v>
+        <v>3690.68</v>
       </c>
       <c r="F70" t="n">
-        <v>80788.06</v>
+        <v>40606.56</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2335,20 +2335,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>동양생명</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4376.39</v>
+        <v>34667.35</v>
       </c>
       <c r="D71" t="n">
-        <v>3483.51</v>
+        <v>3790.53</v>
       </c>
       <c r="E71" t="n">
-        <v>2914.51</v>
+        <v>3101.58</v>
       </c>
       <c r="F71" t="n">
-        <v>90342.16</v>
+        <v>345775.75</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2362,20 +2362,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>LIG넥스원</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>46879.55</v>
+        <v>42899.85</v>
       </c>
       <c r="D72" t="n">
-        <v>3426.07</v>
+        <v>3645.2</v>
       </c>
       <c r="E72" t="n">
-        <v>3916.85</v>
+        <v>2534.49</v>
       </c>
       <c r="F72" t="n">
-        <v>76021.44</v>
+        <v>78329.21000000001</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2389,20 +2389,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HD현대마린솔루션</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>14745.03</v>
+        <v>34627.41</v>
       </c>
       <c r="D73" t="n">
-        <v>3306.95</v>
+        <v>3621.94</v>
       </c>
       <c r="E73" t="n">
-        <v>2552.42</v>
+        <v>2938.25</v>
       </c>
       <c r="F73" t="n">
-        <v>11180.68</v>
+        <v>39999.49</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2416,20 +2416,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>14262.27</v>
+        <v>83779.08</v>
       </c>
       <c r="D74" t="n">
-        <v>3237.64</v>
+        <v>3559.4</v>
       </c>
       <c r="E74" t="n">
-        <v>2581.53</v>
+        <v>3918.63</v>
       </c>
       <c r="F74" t="n">
-        <v>13356.3</v>
+        <v>100939.74</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2443,20 +2443,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>12137.76</v>
+        <v>15282.96</v>
       </c>
       <c r="D75" t="n">
-        <v>3019.39</v>
+        <v>3541.22</v>
       </c>
       <c r="E75" t="n">
-        <v>2718.1</v>
+        <v>2899.39</v>
       </c>
       <c r="F75" t="n">
-        <v>25142.22</v>
+        <v>7342.98</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2470,20 +2470,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>CJ대한통운</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3575.72</v>
+        <v>83538.53</v>
       </c>
       <c r="D76" t="n">
-        <v>3006.52</v>
+        <v>3531.28</v>
       </c>
       <c r="E76" t="n">
-        <v>-1055.72</v>
+        <v>2069.36</v>
       </c>
       <c r="F76" t="n">
-        <v>65984.14</v>
+        <v>80788.06</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2497,20 +2497,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>GS리테일</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>117746.44</v>
+        <v>46879.55</v>
       </c>
       <c r="D77" t="n">
-        <v>2898.97</v>
+        <v>3426.07</v>
       </c>
       <c r="E77" t="n">
-        <v>841.17</v>
+        <v>3916.85</v>
       </c>
       <c r="F77" t="n">
-        <v>71213.37</v>
+        <v>76021.44</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2524,20 +2524,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>롯데렌탈</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>26738.1</v>
+        <v>43152.04</v>
       </c>
       <c r="D78" t="n">
-        <v>2874.97</v>
+        <v>3414.97</v>
       </c>
       <c r="E78" t="n">
-        <v>1070.42</v>
+        <v>488.1</v>
       </c>
       <c r="F78" t="n">
-        <v>66832.8</v>
+        <v>112011.1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2551,20 +2551,20 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>KCC</t>
+          <t>HD현대마린솔루션</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>29357.24</v>
+        <v>14745.03</v>
       </c>
       <c r="D79" t="n">
-        <v>2828.34</v>
+        <v>3306.95</v>
       </c>
       <c r="E79" t="n">
-        <v>20648.95</v>
+        <v>2552.42</v>
       </c>
       <c r="F79" t="n">
-        <v>151265.49</v>
+        <v>11180.68</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2578,20 +2578,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>30914.85</v>
+        <v>17675.96</v>
       </c>
       <c r="D80" t="n">
-        <v>2799.78</v>
+        <v>3282.01</v>
       </c>
       <c r="E80" t="n">
-        <v>3670.39</v>
+        <v>2806.19</v>
       </c>
       <c r="F80" t="n">
-        <v>93434.23</v>
+        <v>67539.56</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2605,20 +2605,20 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>이마트</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>166288.56</v>
+        <v>3978.62</v>
       </c>
       <c r="D81" t="n">
-        <v>2770.72</v>
+        <v>3150.08</v>
       </c>
       <c r="E81" t="n">
-        <v>520.0599999999999</v>
+        <v>2755.98</v>
       </c>
       <c r="F81" t="n">
-        <v>207466.93</v>
+        <v>59512.09</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -2632,20 +2632,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>서울보증보험</t>
+          <t>미스토홀딩스</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>27246.02</v>
+        <v>3434.28</v>
       </c>
       <c r="D82" t="n">
-        <v>2744.37</v>
+        <v>3107.36</v>
       </c>
       <c r="E82" t="n">
-        <v>2109.55</v>
+        <v>3120.43</v>
       </c>
       <c r="F82" t="n">
-        <v>93029.48</v>
+        <v>7944.7</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -2659,20 +2659,20 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>효성</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>5523.08</v>
+        <v>12137.76</v>
       </c>
       <c r="D83" t="n">
-        <v>2703.63</v>
+        <v>3019.39</v>
       </c>
       <c r="E83" t="n">
-        <v>3306.05</v>
+        <v>2718.1</v>
       </c>
       <c r="F83" t="n">
-        <v>33037.02</v>
+        <v>25142.22</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -2686,20 +2686,20 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3770.69</v>
+        <v>3575.72</v>
       </c>
       <c r="D84" t="n">
-        <v>2658.58</v>
+        <v>3006.52</v>
       </c>
       <c r="E84" t="n">
-        <v>2656.02</v>
+        <v>-1055.72</v>
       </c>
       <c r="F84" t="n">
-        <v>70504.62</v>
+        <v>65984.14</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -2713,20 +2713,20 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>GS리테일</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>53071.06</v>
+        <v>117746.44</v>
       </c>
       <c r="D85" t="n">
-        <v>2655.07</v>
+        <v>2898.97</v>
       </c>
       <c r="E85" t="n">
-        <v>1986.36</v>
+        <v>841.17</v>
       </c>
       <c r="F85" t="n">
-        <v>70066.85000000001</v>
+        <v>71213.37</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -2740,20 +2740,20 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SK가스</t>
+          <t>롯데렌탈</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>40564.98</v>
+        <v>26738.1</v>
       </c>
       <c r="D86" t="n">
-        <v>2617.72</v>
+        <v>2874.97</v>
       </c>
       <c r="E86" t="n">
-        <v>1427.91</v>
+        <v>1070.42</v>
       </c>
       <c r="F86" t="n">
-        <v>56380.69</v>
+        <v>66832.8</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -2767,20 +2767,20 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>KCC</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>165124.62</v>
+        <v>29357.24</v>
       </c>
       <c r="D87" t="n">
-        <v>2511.83</v>
+        <v>2828.34</v>
       </c>
       <c r="E87" t="n">
-        <v>2313.3</v>
+        <v>20648.95</v>
       </c>
       <c r="F87" t="n">
-        <v>171912.83</v>
+        <v>151265.49</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -2794,20 +2794,20 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>풍산</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>38491.07</v>
+        <v>3692.7</v>
       </c>
       <c r="D88" t="n">
-        <v>2471.54</v>
+        <v>2816.1</v>
       </c>
       <c r="E88" t="n">
-        <v>1474.06</v>
+        <v>2499.03</v>
       </c>
       <c r="F88" t="n">
-        <v>38473.95</v>
+        <v>68684.23</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -2821,20 +2821,20 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SK바이오팜</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>6506.12</v>
+        <v>30914.85</v>
       </c>
       <c r="D89" t="n">
-        <v>2455.79</v>
+        <v>2799.78</v>
       </c>
       <c r="E89" t="n">
-        <v>2482.68</v>
+        <v>3670.39</v>
       </c>
       <c r="F89" t="n">
-        <v>9554.690000000001</v>
+        <v>93434.23</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -2848,20 +2848,20 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>이마트</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>5596.8</v>
+        <v>166288.56</v>
       </c>
       <c r="D90" t="n">
-        <v>2423.64</v>
+        <v>2770.72</v>
       </c>
       <c r="E90" t="n">
-        <v>2082.76</v>
+        <v>520.0599999999999</v>
       </c>
       <c r="F90" t="n">
-        <v>7986.23</v>
+        <v>207466.93</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -2875,20 +2875,20 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>LIG넥스원</t>
+          <t>서울보증보험</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>32585.75</v>
+        <v>27246.02</v>
       </c>
       <c r="D91" t="n">
-        <v>2412.86</v>
+        <v>2744.37</v>
       </c>
       <c r="E91" t="n">
-        <v>2217.62</v>
+        <v>2109.55</v>
       </c>
       <c r="F91" t="n">
-        <v>59243.52</v>
+        <v>93029.48</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -2902,20 +2902,20 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>신세계</t>
+          <t>영원무역</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>20025.53</v>
+        <v>25074.15</v>
       </c>
       <c r="D92" t="n">
-        <v>2387.6</v>
+        <v>2727.61</v>
       </c>
       <c r="E92" t="n">
-        <v>595.25</v>
+        <v>2636.21</v>
       </c>
       <c r="F92" t="n">
-        <v>93785.89</v>
+        <v>25812.27</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -2929,20 +2929,20 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>강원랜드</t>
+          <t>효성</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>14753.61</v>
+        <v>5523.08</v>
       </c>
       <c r="D93" t="n">
-        <v>2354.71</v>
+        <v>2703.63</v>
       </c>
       <c r="E93" t="n">
-        <v>3072.46</v>
+        <v>3306.05</v>
       </c>
       <c r="F93" t="n">
-        <v>48199.87</v>
+        <v>33037.02</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -2956,20 +2956,20 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>에스원</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>28596.77</v>
+        <v>36252.39</v>
       </c>
       <c r="D94" t="n">
-        <v>2274.64</v>
+        <v>2683.22</v>
       </c>
       <c r="E94" t="n">
-        <v>1905.62</v>
+        <v>1926.99</v>
       </c>
       <c r="F94" t="n">
-        <v>23402.37</v>
+        <v>101972.74</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -2983,20 +2983,20 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>현대백화점</t>
+          <t>BNK금융지주</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>17784.78</v>
+        <v>3770.69</v>
       </c>
       <c r="D95" t="n">
-        <v>2260.67</v>
+        <v>2658.58</v>
       </c>
       <c r="E95" t="n">
-        <v>2031.78</v>
+        <v>2656.02</v>
       </c>
       <c r="F95" t="n">
-        <v>77200.50999999999</v>
+        <v>70504.62</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3010,20 +3010,20 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BGF리테일</t>
+          <t>현대백화점</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>88581.22</v>
+        <v>17955.45</v>
       </c>
       <c r="D96" t="n">
-        <v>2219.57</v>
+        <v>2647.55</v>
       </c>
       <c r="E96" t="n">
-        <v>1740.74</v>
+        <v>1416.93</v>
       </c>
       <c r="F96" t="n">
-        <v>34209.89</v>
+        <v>77964.71000000001</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -3037,20 +3037,20 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>영원무역</t>
+          <t>SK가스</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>21138.86</v>
+        <v>40564.98</v>
       </c>
       <c r="D97" t="n">
-        <v>2151.01</v>
+        <v>2617.72</v>
       </c>
       <c r="E97" t="n">
-        <v>3357.41</v>
+        <v>1427.91</v>
       </c>
       <c r="F97" t="n">
-        <v>28077.3</v>
+        <v>56380.69</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3064,20 +3064,20 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>13909.95</v>
+        <v>165124.62</v>
       </c>
       <c r="D98" t="n">
-        <v>2035.63</v>
+        <v>2511.83</v>
       </c>
       <c r="E98" t="n">
-        <v>1662.56</v>
+        <v>2313.3</v>
       </c>
       <c r="F98" t="n">
-        <v>21009.97</v>
+        <v>171912.83</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3091,20 +3091,20 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>하이트진로</t>
+          <t>풍산</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>23290.35</v>
+        <v>38491.07</v>
       </c>
       <c r="D99" t="n">
-        <v>2015.13</v>
+        <v>2471.54</v>
       </c>
       <c r="E99" t="n">
-        <v>952.13</v>
+        <v>1474.06</v>
       </c>
       <c r="F99" t="n">
-        <v>31882.97</v>
+        <v>38473.95</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -3118,20 +3118,20 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>금호석유화학</t>
+          <t>HDC현대산업개발</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>45719.79</v>
+        <v>40892.93</v>
       </c>
       <c r="D100" t="n">
-        <v>1981.21</v>
+        <v>2459.92</v>
       </c>
       <c r="E100" t="n">
-        <v>1757.31</v>
+        <v>1647.83</v>
       </c>
       <c r="F100" t="n">
-        <v>46201.49</v>
+        <v>72542.24000000001</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -3145,20 +3145,20 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>현대오토에버</t>
+          <t>SK바이오팜</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>29434.44</v>
+        <v>6506.12</v>
       </c>
       <c r="D101" t="n">
-        <v>1968.51</v>
+        <v>2455.79</v>
       </c>
       <c r="E101" t="n">
-        <v>1626.95</v>
+        <v>2482.68</v>
       </c>
       <c r="F101" t="n">
-        <v>29791.66</v>
+        <v>9554.690000000001</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -3172,20 +3172,20 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CJ제일제당</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>72811.41</v>
+        <v>5596.8</v>
       </c>
       <c r="D102" t="n">
-        <v>1856.31</v>
+        <v>2423.64</v>
       </c>
       <c r="E102" t="n">
-        <v>-5896.05</v>
+        <v>2082.76</v>
       </c>
       <c r="F102" t="n">
-        <v>106127.75</v>
+        <v>7986.23</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -3199,20 +3199,20 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>HDC현대산업개발</t>
+          <t>신세계</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>42113.73</v>
+        <v>20025.53</v>
       </c>
       <c r="D103" t="n">
-        <v>1846.95</v>
+        <v>2387.6</v>
       </c>
       <c r="E103" t="n">
-        <v>1587.78</v>
+        <v>595.25</v>
       </c>
       <c r="F103" t="n">
-        <v>71334.16</v>
+        <v>93785.89</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -3226,20 +3226,20 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>대한해운</t>
+          <t>강원랜드</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>8566.25</v>
+        <v>14753.61</v>
       </c>
       <c r="D104" t="n">
-        <v>1814.1</v>
+        <v>2354.71</v>
       </c>
       <c r="E104" t="n">
-        <v>1486.71</v>
+        <v>3072.46</v>
       </c>
       <c r="F104" t="n">
-        <v>22826.67</v>
+        <v>48199.87</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -3253,20 +3253,20 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>에스엘</t>
+          <t>S-Oil</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>26820.77</v>
+        <v>338960.41</v>
       </c>
       <c r="D105" t="n">
-        <v>1800.4</v>
+        <v>2309.03</v>
       </c>
       <c r="E105" t="n">
-        <v>2606.21</v>
+        <v>1869.07</v>
       </c>
       <c r="F105" t="n">
-        <v>24099.74</v>
+        <v>265200.56</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -3280,20 +3280,20 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>89891.25</v>
+        <v>47501.15</v>
       </c>
       <c r="D106" t="n">
-        <v>1795.97</v>
+        <v>2293.18</v>
       </c>
       <c r="E106" t="n">
-        <v>999.77</v>
+        <v>977.03</v>
       </c>
       <c r="F106" t="n">
-        <v>47388.73</v>
+        <v>68784.28999999999</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -3307,20 +3307,20 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>오리온</t>
+          <t>에스원</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>10976.13</v>
+        <v>28596.77</v>
       </c>
       <c r="D107" t="n">
-        <v>1784.78</v>
+        <v>2274.64</v>
       </c>
       <c r="E107" t="n">
-        <v>3555.42</v>
+        <v>1905.62</v>
       </c>
       <c r="F107" t="n">
-        <v>16531.45</v>
+        <v>23402.37</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -3334,20 +3334,20 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>교보증권</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>31683.52</v>
+        <v>71141.53999999999</v>
       </c>
       <c r="D108" t="n">
-        <v>1677.37</v>
+        <v>2260.22</v>
       </c>
       <c r="E108" t="n">
-        <v>1371.03</v>
+        <v>1078.99</v>
       </c>
       <c r="F108" t="n">
-        <v>152533.09</v>
+        <v>40876.36</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -3361,20 +3361,20 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>아이에스동서</t>
+          <t>BGF리테일</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9514.799999999999</v>
+        <v>88581.22</v>
       </c>
       <c r="D109" t="n">
-        <v>1660.74</v>
+        <v>2219.57</v>
       </c>
       <c r="E109" t="n">
-        <v>-1623.32</v>
+        <v>1740.74</v>
       </c>
       <c r="F109" t="n">
-        <v>29895.06</v>
+        <v>34209.89</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -3388,20 +3388,20 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>LX세미콘</t>
+          <t>아모레퍼시픽</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>18656.22</v>
+        <v>26537.26</v>
       </c>
       <c r="D110" t="n">
-        <v>1641.17</v>
+        <v>2125.15</v>
       </c>
       <c r="E110" t="n">
-        <v>1291.69</v>
+        <v>3179.2</v>
       </c>
       <c r="F110" t="n">
-        <v>14851.86</v>
+        <v>56252.44</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -3415,20 +3415,20 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>에스엘</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>10746.19</v>
+        <v>29690.29</v>
       </c>
       <c r="D111" t="n">
-        <v>1581.86</v>
+        <v>2073.32</v>
       </c>
       <c r="E111" t="n">
-        <v>1722.95</v>
+        <v>2069.5</v>
       </c>
       <c r="F111" t="n">
-        <v>13490.33</v>
+        <v>26146.19</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -3442,20 +3442,20 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>20182.27</v>
+        <v>13909.95</v>
       </c>
       <c r="D112" t="n">
-        <v>1535.19</v>
+        <v>2035.63</v>
       </c>
       <c r="E112" t="n">
-        <v>1065.76</v>
+        <v>1662.56</v>
       </c>
       <c r="F112" t="n">
-        <v>14784.9</v>
+        <v>21009.97</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -3469,20 +3469,20 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>시프트업</t>
+          <t>한국앤컴퍼니</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2240.85</v>
+        <v>11007.84</v>
       </c>
       <c r="D113" t="n">
-        <v>1526.76</v>
+        <v>2015.15</v>
       </c>
       <c r="E113" t="n">
-        <v>1479.73</v>
+        <v>1587.63</v>
       </c>
       <c r="F113" t="n">
-        <v>8038.32</v>
+        <v>29550.88</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -3496,20 +3496,20 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>대상</t>
+          <t>금호석유화학</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>34850.2</v>
+        <v>45719.79</v>
       </c>
       <c r="D114" t="n">
-        <v>1495.06</v>
+        <v>1981.21</v>
       </c>
       <c r="E114" t="n">
-        <v>1113.43</v>
+        <v>1757.31</v>
       </c>
       <c r="F114" t="n">
-        <v>30822.91</v>
+        <v>46201.49</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -3523,20 +3523,20 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>경동나비엔</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>12468.55</v>
+        <v>29434.44</v>
       </c>
       <c r="D115" t="n">
-        <v>1492.64</v>
+        <v>1968.51</v>
       </c>
       <c r="E115" t="n">
-        <v>1357.22</v>
+        <v>1626.95</v>
       </c>
       <c r="F115" t="n">
-        <v>10162.34</v>
+        <v>29791.66</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -3550,20 +3550,20 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>흥국화재</t>
+          <t>오리온</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>33740.16</v>
+        <v>11458.38</v>
       </c>
       <c r="D116" t="n">
-        <v>1487.79</v>
+        <v>1868.17</v>
       </c>
       <c r="E116" t="n">
-        <v>1067.22</v>
+        <v>4003.12</v>
       </c>
       <c r="F116" t="n">
-        <v>128946.89</v>
+        <v>19453.14</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -3577,20 +3577,20 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>신영증권</t>
+          <t>CJ제일제당</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>24057.52</v>
+        <v>72811.41</v>
       </c>
       <c r="D117" t="n">
-        <v>1455.17</v>
+        <v>1856.31</v>
       </c>
       <c r="E117" t="n">
-        <v>1181.51</v>
+        <v>-5896.05</v>
       </c>
       <c r="F117" t="n">
-        <v>98188.64999999999</v>
+        <v>106127.75</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -3604,20 +3604,20 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>세방전지</t>
+          <t>대한해운</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>15820.33</v>
+        <v>8566.25</v>
       </c>
       <c r="D118" t="n">
-        <v>1424.97</v>
+        <v>1814.1</v>
       </c>
       <c r="E118" t="n">
-        <v>1494.72</v>
+        <v>1486.71</v>
       </c>
       <c r="F118" t="n">
-        <v>17638.03</v>
+        <v>22826.67</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -3631,20 +3631,20 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>한국앤컴퍼니</t>
+          <t>산일전기</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>9987.18</v>
+        <v>5019.46</v>
       </c>
       <c r="D119" t="n">
-        <v>1410.38</v>
+        <v>1790.4</v>
       </c>
       <c r="E119" t="n">
-        <v>945.1</v>
+        <v>1491.41</v>
       </c>
       <c r="F119" t="n">
-        <v>31730.56</v>
+        <v>6811.01</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -3658,20 +3658,20 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>한전KPS</t>
+          <t>하이트진로</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>15452.56</v>
+        <v>22404.32</v>
       </c>
       <c r="D120" t="n">
-        <v>1393.76</v>
+        <v>1723.46</v>
       </c>
       <c r="E120" t="n">
-        <v>1237.96</v>
+        <v>480.04</v>
       </c>
       <c r="F120" t="n">
-        <v>16877.6</v>
+        <v>30334.13</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -3685,20 +3685,20 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>효성티앤씨</t>
+          <t>교보증권</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>43251.72</v>
+        <v>31683.52</v>
       </c>
       <c r="D121" t="n">
-        <v>1392.14</v>
+        <v>1677.37</v>
       </c>
       <c r="E121" t="n">
-        <v>1437.46</v>
+        <v>1371.03</v>
       </c>
       <c r="F121" t="n">
-        <v>22969.8</v>
+        <v>152533.09</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -3712,20 +3712,20 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>코스맥스</t>
+          <t>현대위아</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>13576.6</v>
+        <v>72787.97</v>
       </c>
       <c r="D122" t="n">
-        <v>1386.79</v>
+        <v>1676.1</v>
       </c>
       <c r="E122" t="n">
-        <v>1066.54</v>
+        <v>-184.68</v>
       </c>
       <c r="F122" t="n">
-        <v>11889.73</v>
+        <v>55756.53</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -3739,20 +3739,20 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이에스동서</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>34084.92</v>
+        <v>9514.799999999999</v>
       </c>
       <c r="D123" t="n">
-        <v>1373.86</v>
+        <v>1660.74</v>
       </c>
       <c r="E123" t="n">
-        <v>1210.02</v>
+        <v>-1623.32</v>
       </c>
       <c r="F123" t="n">
-        <v>173152.31</v>
+        <v>29895.06</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -3766,20 +3766,20 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>미스토홀딩스</t>
+          <t>한국타이어앤테크놀로지</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1628.82</v>
+        <v>36484.38</v>
       </c>
       <c r="D124" t="n">
-        <v>1373.36</v>
+        <v>1624.95</v>
       </c>
       <c r="E124" t="n">
-        <v>1289.77</v>
+        <v>9907.75</v>
       </c>
       <c r="F124" t="n">
-        <v>8460.629999999999</v>
+        <v>88571.17</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -3793,20 +3793,20 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>32985.69</v>
+        <v>1745.8</v>
       </c>
       <c r="D125" t="n">
-        <v>1370.87</v>
+        <v>1605.6</v>
       </c>
       <c r="E125" t="n">
-        <v>7389.01</v>
+        <v>1905.17</v>
       </c>
       <c r="F125" t="n">
-        <v>84540.89</v>
+        <v>38519.64</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -3820,20 +3820,20 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>CJ</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2460.9</v>
+        <v>10746.19</v>
       </c>
       <c r="D126" t="n">
-        <v>1362.63</v>
+        <v>1581.86</v>
       </c>
       <c r="E126" t="n">
-        <v>2253.35</v>
+        <v>1722.95</v>
       </c>
       <c r="F126" t="n">
-        <v>34703.66</v>
+        <v>13490.33</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -3847,20 +3847,20 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>한세실업</t>
+          <t>동원산업</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>17190.24</v>
+        <v>11062.5</v>
       </c>
       <c r="D127" t="n">
-        <v>1355.28</v>
+        <v>1556.56</v>
       </c>
       <c r="E127" t="n">
-        <v>800.01</v>
+        <v>1278.59</v>
       </c>
       <c r="F127" t="n">
-        <v>11432.63</v>
+        <v>36130.59</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -3874,20 +3874,20 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>코스맥스</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2404.29</v>
+        <v>15264.15</v>
       </c>
       <c r="D128" t="n">
-        <v>1354.23</v>
+        <v>1545.78</v>
       </c>
       <c r="E128" t="n">
-        <v>1359.64</v>
+        <v>1311.61</v>
       </c>
       <c r="F128" t="n">
-        <v>47399.91</v>
+        <v>13649.39</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -3901,20 +3901,20 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>롯데지주</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3391.18</v>
+        <v>20182.27</v>
       </c>
       <c r="D129" t="n">
-        <v>1341.88</v>
+        <v>1535.19</v>
       </c>
       <c r="E129" t="n">
-        <v>754.03</v>
+        <v>1065.76</v>
       </c>
       <c r="F129" t="n">
-        <v>90920.25999999999</v>
+        <v>14784.9</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -3928,20 +3928,20 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>농심</t>
+          <t>시프트업</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>27347.14</v>
+        <v>2240.85</v>
       </c>
       <c r="D130" t="n">
-        <v>1338.22</v>
+        <v>1526.76</v>
       </c>
       <c r="E130" t="n">
-        <v>1388.78</v>
+        <v>1479.73</v>
       </c>
       <c r="F130" t="n">
-        <v>32321.21</v>
+        <v>8038.32</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -3955,20 +3955,20 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>KG스틸</t>
+          <t>계룡건설</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>29263.88</v>
+        <v>20235.46</v>
       </c>
       <c r="D131" t="n">
-        <v>1335.13</v>
+        <v>1525.02</v>
       </c>
       <c r="E131" t="n">
-        <v>1194.31</v>
+        <v>1132.15</v>
       </c>
       <c r="F131" t="n">
-        <v>29746.49</v>
+        <v>22872.78</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -3982,20 +3982,20 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>케이뱅크</t>
+          <t>현대엘리베이터</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>12285.01</v>
+        <v>16071</v>
       </c>
       <c r="D132" t="n">
-        <v>1329.67</v>
+        <v>1508.32</v>
       </c>
       <c r="E132" t="n">
-        <v>1280.53</v>
+        <v>3111.36</v>
       </c>
       <c r="F132" t="n">
-        <v>311833.99</v>
+        <v>27628.05</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -4009,20 +4009,20 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>대상</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>11141.23</v>
+        <v>35288.56</v>
       </c>
       <c r="D133" t="n">
-        <v>1327.01</v>
+        <v>1505.19</v>
       </c>
       <c r="E133" t="n">
-        <v>1305.88</v>
+        <v>-2855.56</v>
       </c>
       <c r="F133" t="n">
-        <v>14128.13</v>
+        <v>30613.98</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -4036,20 +4036,20 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>동원산업</t>
+          <t>한국콜마</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>10794.15</v>
+        <v>11927.52</v>
       </c>
       <c r="D134" t="n">
-        <v>1285.51</v>
+        <v>1495.33</v>
       </c>
       <c r="E134" t="n">
-        <v>1142.36</v>
+        <v>1142.71</v>
       </c>
       <c r="F134" t="n">
-        <v>31661.57</v>
+        <v>15290.03</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -4063,20 +4063,20 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>흥국화재</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>10596.69</v>
+        <v>33740.16</v>
       </c>
       <c r="D135" t="n">
-        <v>1223.36</v>
+        <v>1487.79</v>
       </c>
       <c r="E135" t="n">
-        <v>1390.49</v>
+        <v>1067.22</v>
       </c>
       <c r="F135" t="n">
-        <v>14107.32</v>
+        <v>128946.89</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -4090,20 +4090,20 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>영원무역홀딩스</t>
+          <t>CJ</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1514.61</v>
+        <v>2621.58</v>
       </c>
       <c r="D136" t="n">
-        <v>1220.16</v>
+        <v>1464.83</v>
       </c>
       <c r="E136" t="n">
-        <v>1241.82</v>
+        <v>1355.11</v>
       </c>
       <c r="F136" t="n">
-        <v>7242.69</v>
+        <v>33855.18</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -4117,20 +4117,20 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>오뚜기</t>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>29267.67</v>
+        <v>24057.52</v>
       </c>
       <c r="D137" t="n">
-        <v>1211.42</v>
+        <v>1455.17</v>
       </c>
       <c r="E137" t="n">
-        <v>970.6799999999999</v>
+        <v>1181.51</v>
       </c>
       <c r="F137" t="n">
-        <v>25617.26</v>
+        <v>98188.64999999999</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -4144,20 +4144,20 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>HL홀딩스</t>
+          <t>세방전지</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>9474.16</v>
+        <v>15820.33</v>
       </c>
       <c r="D138" t="n">
-        <v>1193.99</v>
+        <v>1424.97</v>
       </c>
       <c r="E138" t="n">
-        <v>373.36</v>
+        <v>1494.72</v>
       </c>
       <c r="F138" t="n">
-        <v>21787.92</v>
+        <v>17638.03</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -4171,20 +4171,20 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>한솔케미칼</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>7230.01</v>
+        <v>6831.82</v>
       </c>
       <c r="D139" t="n">
-        <v>1183.98</v>
+        <v>1399.96</v>
       </c>
       <c r="E139" t="n">
-        <v>1070.95</v>
+        <v>1387.79</v>
       </c>
       <c r="F139" t="n">
-        <v>5287.99</v>
+        <v>12663.1</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -4198,20 +4198,20 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>한솔케미칼</t>
+          <t>한전KPS</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>5848.51</v>
+        <v>15452.56</v>
       </c>
       <c r="D140" t="n">
-        <v>1157.64</v>
+        <v>1393.76</v>
       </c>
       <c r="E140" t="n">
-        <v>953.88</v>
+        <v>1237.96</v>
       </c>
       <c r="F140" t="n">
-        <v>11527.45</v>
+        <v>16877.6</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -4225,20 +4225,20 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>미래에셋생명</t>
+          <t>효성티앤씨</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>46539.62</v>
+        <v>43251.72</v>
       </c>
       <c r="D141" t="n">
-        <v>1149.39</v>
+        <v>1392.14</v>
       </c>
       <c r="E141" t="n">
-        <v>1250.39</v>
+        <v>1437.46</v>
       </c>
       <c r="F141" t="n">
-        <v>324044.39</v>
+        <v>22969.8</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -4252,20 +4252,20 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>서연이화</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>17970.17</v>
+        <v>34084.92</v>
       </c>
       <c r="D142" t="n">
-        <v>1128.03</v>
+        <v>1373.86</v>
       </c>
       <c r="E142" t="n">
-        <v>1504.02</v>
+        <v>1210.02</v>
       </c>
       <c r="F142" t="n">
-        <v>18473.82</v>
+        <v>173152.31</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -4279,20 +4279,20 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>한진칼</t>
+          <t>한세실업</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1355.74</v>
+        <v>17190.24</v>
       </c>
       <c r="D143" t="n">
-        <v>1110.76</v>
+        <v>1355.28</v>
       </c>
       <c r="E143" t="n">
-        <v>1930.07</v>
+        <v>800.01</v>
       </c>
       <c r="F143" t="n">
-        <v>32090.19</v>
+        <v>11432.63</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -4306,20 +4306,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>유한양행</t>
+          <t>iM금융지주</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>21056.61</v>
+        <v>2404.29</v>
       </c>
       <c r="D144" t="n">
-        <v>1101.96</v>
+        <v>1354.23</v>
       </c>
       <c r="E144" t="n">
-        <v>2095.66</v>
+        <v>1359.64</v>
       </c>
       <c r="F144" t="n">
-        <v>27138.37</v>
+        <v>47399.91</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -4333,20 +4333,20 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SNT모티브</t>
+          <t>롯데지주</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>9987.389999999999</v>
+        <v>3391.18</v>
       </c>
       <c r="D145" t="n">
-        <v>1091.61</v>
+        <v>1341.88</v>
       </c>
       <c r="E145" t="n">
-        <v>760.4</v>
+        <v>754.03</v>
       </c>
       <c r="F145" t="n">
-        <v>12681.8</v>
+        <v>90920.25999999999</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -4360,20 +4360,20 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>넥센타이어</t>
+          <t>농심</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>21326.25</v>
+        <v>27347.14</v>
       </c>
       <c r="D146" t="n">
-        <v>1089.63</v>
+        <v>1338.22</v>
       </c>
       <c r="E146" t="n">
-        <v>1493.9</v>
+        <v>1388.78</v>
       </c>
       <c r="F146" t="n">
-        <v>35805.02</v>
+        <v>32321.21</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -4387,20 +4387,20 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>INVENI</t>
+          <t>KG스틸</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1728.82</v>
+        <v>29263.88</v>
       </c>
       <c r="D147" t="n">
-        <v>1078.85</v>
+        <v>1335.13</v>
       </c>
       <c r="E147" t="n">
-        <v>857.29</v>
+        <v>1194.31</v>
       </c>
       <c r="F147" t="n">
-        <v>8289.09</v>
+        <v>29746.49</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -4414,20 +4414,20 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>DN오토모티브</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>9862.799999999999</v>
+        <v>12285.01</v>
       </c>
       <c r="D148" t="n">
-        <v>1071.15</v>
+        <v>1329.67</v>
       </c>
       <c r="E148" t="n">
-        <v>689.6799999999999</v>
+        <v>1280.53</v>
       </c>
       <c r="F148" t="n">
-        <v>19240.2</v>
+        <v>311833.99</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -4441,20 +4441,20 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>31182.23</v>
+        <v>11141.23</v>
       </c>
       <c r="D149" t="n">
-        <v>1069.43</v>
+        <v>1327.01</v>
       </c>
       <c r="E149" t="n">
-        <v>762.59</v>
+        <v>1305.88</v>
       </c>
       <c r="F149" t="n">
-        <v>32302.89</v>
+        <v>14128.13</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -4468,20 +4468,20 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>쿠쿠홈시스</t>
+          <t>경동나비엔</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>7431.22</v>
+        <v>12635.45</v>
       </c>
       <c r="D150" t="n">
-        <v>1050.08</v>
+        <v>1317.96</v>
       </c>
       <c r="E150" t="n">
-        <v>1115.54</v>
+        <v>822.85</v>
       </c>
       <c r="F150" t="n">
-        <v>9414.129999999999</v>
+        <v>10845.89</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -4495,20 +4495,20 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>KSS해운</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>5178.86</v>
+        <v>13710.57</v>
       </c>
       <c r="D151" t="n">
-        <v>1040.71</v>
+        <v>1300.66</v>
       </c>
       <c r="E151" t="n">
-        <v>573.85</v>
+        <v>1737.53</v>
       </c>
       <c r="F151" t="n">
-        <v>18909.83</v>
+        <v>16956.95</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -4522,20 +4522,20 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>현대그린푸드</t>
+          <t>한일시멘트</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>22742.22</v>
+        <v>10110.96</v>
       </c>
       <c r="D152" t="n">
-        <v>1021.74</v>
+        <v>1257.39</v>
       </c>
       <c r="E152" t="n">
-        <v>819.58</v>
+        <v>857.46</v>
       </c>
       <c r="F152" t="n">
-        <v>10111.77</v>
+        <v>30007.28</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -4549,20 +4549,20 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>롯데칠성</t>
+          <t>서연이화</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>25669.7</v>
+        <v>19254.2</v>
       </c>
       <c r="D153" t="n">
-        <v>1020.95</v>
+        <v>1233.56</v>
       </c>
       <c r="E153" t="n">
-        <v>484.61</v>
+        <v>175.7</v>
       </c>
       <c r="F153" t="n">
-        <v>34103.71</v>
+        <v>18152.93</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -4576,20 +4576,20 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>NHN</t>
+          <t>영원무역홀딩스</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3743.93</v>
+        <v>1514.61</v>
       </c>
       <c r="D154" t="n">
-        <v>1004.22</v>
+        <v>1220.16</v>
       </c>
       <c r="E154" t="n">
-        <v>218.5</v>
+        <v>1241.82</v>
       </c>
       <c r="F154" t="n">
-        <v>18630.58</v>
+        <v>7242.69</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -4603,20 +4603,20 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>제일기획</t>
+          <t>HL홀딩스</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>14156.23</v>
+        <v>9474.16</v>
       </c>
       <c r="D155" t="n">
-        <v>972</v>
+        <v>1193.99</v>
       </c>
       <c r="E155" t="n">
-        <v>1059.79</v>
+        <v>373.36</v>
       </c>
       <c r="F155" t="n">
-        <v>12749.87</v>
+        <v>21787.92</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -4630,20 +4630,20 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>JW중외제약</t>
+          <t>미래에셋생명</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>7671.5</v>
+        <v>46539.62</v>
       </c>
       <c r="D156" t="n">
-        <v>966.3</v>
+        <v>1149.39</v>
       </c>
       <c r="E156" t="n">
-        <v>613.1</v>
+        <v>1250.39</v>
       </c>
       <c r="F156" t="n">
-        <v>5959.35</v>
+        <v>324044.39</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -4657,20 +4657,20 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>SK케미칼</t>
+          <t>한온시스템</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>14403.81</v>
+        <v>39300.4</v>
       </c>
       <c r="D157" t="n">
-        <v>957.13</v>
+        <v>1118.59</v>
       </c>
       <c r="E157" t="n">
-        <v>689.76</v>
+        <v>-2169.58</v>
       </c>
       <c r="F157" t="n">
-        <v>23232.52</v>
+        <v>71519.27</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -4684,20 +4684,20 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>SNT에너지</t>
+          <t>유한양행</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>4991.46</v>
+        <v>21056.61</v>
       </c>
       <c r="D158" t="n">
-        <v>955.37</v>
+        <v>1101.96</v>
       </c>
       <c r="E158" t="n">
-        <v>741.41</v>
+        <v>2095.66</v>
       </c>
       <c r="F158" t="n">
-        <v>5261.4</v>
+        <v>27138.37</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -4711,20 +4711,20 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>SNT모티브</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1102.07</v>
+        <v>9987.389999999999</v>
       </c>
       <c r="D159" t="n">
-        <v>911.65</v>
+        <v>1091.61</v>
       </c>
       <c r="E159" t="n">
-        <v>1993.08</v>
+        <v>760.4</v>
       </c>
       <c r="F159" t="n">
-        <v>37442.7</v>
+        <v>12681.8</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -4738,20 +4738,20 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>NICE평가정보</t>
+          <t>쿠쿠홈시스</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>4759.14</v>
+        <v>8066.44</v>
       </c>
       <c r="D160" t="n">
-        <v>906.97</v>
+        <v>1085.42</v>
       </c>
       <c r="E160" t="n">
-        <v>689.2</v>
+        <v>1187.4</v>
       </c>
       <c r="F160" t="n">
-        <v>5568.22</v>
+        <v>10494.67</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -4765,20 +4765,20 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>유안타증권</t>
+          <t>INVENI</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>26720.77</v>
+        <v>1728.82</v>
       </c>
       <c r="D161" t="n">
-        <v>906.36</v>
+        <v>1078.85</v>
       </c>
       <c r="E161" t="n">
-        <v>902.75</v>
+        <v>857.29</v>
       </c>
       <c r="F161" t="n">
-        <v>161325.78</v>
+        <v>8289.09</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -4792,20 +4792,20 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>명인제약</t>
+          <t>DN오토모티브</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2695.86</v>
+        <v>9862.799999999999</v>
       </c>
       <c r="D162" t="n">
-        <v>900.58</v>
+        <v>1071.15</v>
       </c>
       <c r="E162" t="n">
-        <v>661.52</v>
+        <v>689.6799999999999</v>
       </c>
       <c r="F162" t="n">
-        <v>5729.23</v>
+        <v>19240.2</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -4819,20 +4819,20 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>롯데웰푸드</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>32828.57</v>
+        <v>31182.23</v>
       </c>
       <c r="D163" t="n">
-        <v>842.35</v>
+        <v>1069.43</v>
       </c>
       <c r="E163" t="n">
-        <v>661.52</v>
+        <v>762.59</v>
       </c>
       <c r="F163" t="n">
-        <v>41168.64</v>
+        <v>32302.89</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -4846,20 +4846,20 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>SNT다이내믹스</t>
+          <t>LX세미콘</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>6051.36</v>
+        <v>16390.71</v>
       </c>
       <c r="D164" t="n">
-        <v>833.74</v>
+        <v>1055.77</v>
       </c>
       <c r="E164" t="n">
-        <v>598.92</v>
+        <v>824.99</v>
       </c>
       <c r="F164" t="n">
-        <v>11983.81</v>
+        <v>13862.72</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -4873,20 +4873,20 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>AJ네트웍스</t>
+          <t>KSS해운</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>6116.78</v>
+        <v>5178.86</v>
       </c>
       <c r="D165" t="n">
-        <v>831.51</v>
+        <v>1040.71</v>
       </c>
       <c r="E165" t="n">
-        <v>249.99</v>
+        <v>573.85</v>
       </c>
       <c r="F165" t="n">
-        <v>16191.13</v>
+        <v>18909.83</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -4900,20 +4900,20 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TKG휴켐스</t>
+          <t>현대그린푸드</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>11785.03</v>
+        <v>22742.22</v>
       </c>
       <c r="D166" t="n">
-        <v>828.05</v>
+        <v>1021.74</v>
       </c>
       <c r="E166" t="n">
-        <v>805.04</v>
+        <v>819.58</v>
       </c>
       <c r="F166" t="n">
-        <v>10689.74</v>
+        <v>10111.77</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -4927,20 +4927,20 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>한국단자</t>
+          <t>롯데칠성</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>11706.86</v>
+        <v>25669.7</v>
       </c>
       <c r="D167" t="n">
-        <v>825.5700000000001</v>
+        <v>1020.95</v>
       </c>
       <c r="E167" t="n">
-        <v>670.95</v>
+        <v>484.61</v>
       </c>
       <c r="F167" t="n">
-        <v>12653.33</v>
+        <v>34103.71</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -4954,20 +4954,20 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>NHN</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>10664.95</v>
+        <v>3743.93</v>
       </c>
       <c r="D168" t="n">
-        <v>816.11</v>
+        <v>1004.22</v>
       </c>
       <c r="E168" t="n">
-        <v>232.42</v>
+        <v>218.5</v>
       </c>
       <c r="F168" t="n">
-        <v>50535.26</v>
+        <v>18630.58</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -4981,20 +4981,20 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>동원시스템즈</t>
+          <t>화승코퍼레이션</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>12301.44</v>
+        <v>4888.31</v>
       </c>
       <c r="D169" t="n">
-        <v>811.66</v>
+        <v>999.0599999999999</v>
       </c>
       <c r="E169" t="n">
-        <v>865.14</v>
+        <v>922.66</v>
       </c>
       <c r="F169" t="n">
-        <v>14835.59</v>
+        <v>5612.99</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -5008,20 +5008,20 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>종근당</t>
+          <t>제일기획</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>16811.92</v>
+        <v>14156.23</v>
       </c>
       <c r="D170" t="n">
-        <v>801.08</v>
+        <v>972</v>
       </c>
       <c r="E170" t="n">
-        <v>868.0700000000001</v>
+        <v>1059.79</v>
       </c>
       <c r="F170" t="n">
-        <v>17869.38</v>
+        <v>12749.87</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -5035,20 +5035,20 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>SPC삼립</t>
+          <t>JW중외제약</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>16470.64</v>
+        <v>7671.5</v>
       </c>
       <c r="D171" t="n">
-        <v>801.01</v>
+        <v>966.3</v>
       </c>
       <c r="E171" t="n">
-        <v>768.87</v>
+        <v>613.1</v>
       </c>
       <c r="F171" t="n">
-        <v>9208.059999999999</v>
+        <v>5959.35</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -5062,20 +5062,20 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>7187.29</v>
+        <v>11406.2</v>
       </c>
       <c r="D172" t="n">
-        <v>784.8</v>
+        <v>958.21</v>
       </c>
       <c r="E172" t="n">
-        <v>652.48</v>
+        <v>986.53</v>
       </c>
       <c r="F172" t="n">
-        <v>6871.52</v>
+        <v>19353.88</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -5089,20 +5089,20 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>삼양사</t>
+          <t>SK케미칼</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>19663.33</v>
+        <v>14403.81</v>
       </c>
       <c r="D173" t="n">
-        <v>774.87</v>
+        <v>957.13</v>
       </c>
       <c r="E173" t="n">
-        <v>892.8</v>
+        <v>689.76</v>
       </c>
       <c r="F173" t="n">
-        <v>25748.88</v>
+        <v>23232.52</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -5116,20 +5116,20 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>현대홈쇼핑</t>
+          <t>SNT에너지</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>10898.89</v>
+        <v>4991.46</v>
       </c>
       <c r="D174" t="n">
-        <v>773.33</v>
+        <v>955.37</v>
       </c>
       <c r="E174" t="n">
-        <v>946.41</v>
+        <v>741.41</v>
       </c>
       <c r="F174" t="n">
-        <v>18981.43</v>
+        <v>5261.4</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -5143,20 +5143,20 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>현대코퍼레이션</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>48450.25</v>
+        <v>21500.89</v>
       </c>
       <c r="D175" t="n">
-        <v>768.65</v>
+        <v>910.37</v>
       </c>
       <c r="E175" t="n">
-        <v>1215.73</v>
+        <v>510.71</v>
       </c>
       <c r="F175" t="n">
-        <v>16474.43</v>
+        <v>24212.92</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -5170,20 +5170,20 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>롯데정밀화학</t>
+          <t>NICE평가정보</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>17503.45</v>
+        <v>4759.14</v>
       </c>
       <c r="D176" t="n">
-        <v>745.12</v>
+        <v>906.97</v>
       </c>
       <c r="E176" t="n">
-        <v>1030.29</v>
+        <v>689.2</v>
       </c>
       <c r="F176" t="n">
-        <v>25389.86</v>
+        <v>5568.22</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -5197,20 +5197,20 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>아세아시멘트</t>
+          <t>유안타증권</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>5078.56</v>
+        <v>26720.77</v>
       </c>
       <c r="D177" t="n">
-        <v>731.24</v>
+        <v>906.36</v>
       </c>
       <c r="E177" t="n">
-        <v>459.87</v>
+        <v>902.75</v>
       </c>
       <c r="F177" t="n">
-        <v>12321.47</v>
+        <v>161325.78</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -5224,20 +5224,20 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>빙그레</t>
+          <t>명인제약</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>13124.34</v>
+        <v>2695.86</v>
       </c>
       <c r="D178" t="n">
-        <v>730.79</v>
+        <v>900.58</v>
       </c>
       <c r="E178" t="n">
-        <v>519.89</v>
+        <v>661.52</v>
       </c>
       <c r="F178" t="n">
-        <v>10157.36</v>
+        <v>5729.23</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -5251,20 +5251,20 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>SNT홀딩스</t>
+          <t>오뚜기</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>765.9</v>
+        <v>29886.55</v>
       </c>
       <c r="D179" t="n">
-        <v>727.72</v>
+        <v>893.8099999999999</v>
       </c>
       <c r="E179" t="n">
-        <v>1374.78</v>
+        <v>617.72</v>
       </c>
       <c r="F179" t="n">
-        <v>6049.49</v>
+        <v>25944.56</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -5278,20 +5278,20 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>12022.05</v>
+        <v>178001.26</v>
       </c>
       <c r="D180" t="n">
-        <v>715.3200000000001</v>
+        <v>892.35</v>
       </c>
       <c r="E180" t="n">
-        <v>791.6</v>
+        <v>-409.17</v>
       </c>
       <c r="F180" t="n">
-        <v>14131.02</v>
+        <v>314554.55</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -5305,20 +5305,20 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>덴티움</t>
+          <t>롯데웰푸드</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>3207.23</v>
+        <v>32828.57</v>
       </c>
       <c r="D181" t="n">
-        <v>706.26</v>
+        <v>842.35</v>
       </c>
       <c r="E181" t="n">
-        <v>267.33</v>
+        <v>661.52</v>
       </c>
       <c r="F181" t="n">
-        <v>7373.13</v>
+        <v>41168.64</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -5332,20 +5332,20 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>세아베스틸지주</t>
+          <t>SNT다이내믹스</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>883.78</v>
+        <v>6051.36</v>
       </c>
       <c r="D182" t="n">
-        <v>702.03</v>
+        <v>833.74</v>
       </c>
       <c r="E182" t="n">
-        <v>643.42</v>
+        <v>598.92</v>
       </c>
       <c r="F182" t="n">
-        <v>18317.64</v>
+        <v>11983.81</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -5359,20 +5359,20 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>HD현대마린엔진</t>
+          <t>한국단자</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>3798.48</v>
+        <v>11706.86</v>
       </c>
       <c r="D183" t="n">
-        <v>684.52</v>
+        <v>825.5700000000001</v>
       </c>
       <c r="E183" t="n">
-        <v>1573.79</v>
+        <v>670.95</v>
       </c>
       <c r="F183" t="n">
-        <v>7833.44</v>
+        <v>12653.33</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -5386,20 +5386,20 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>케이카</t>
+          <t>동원시스템즈</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>23015.3</v>
+        <v>12301.44</v>
       </c>
       <c r="D184" t="n">
-        <v>681.09</v>
+        <v>811.66</v>
       </c>
       <c r="E184" t="n">
-        <v>439.65</v>
+        <v>865.14</v>
       </c>
       <c r="F184" t="n">
-        <v>5248.48</v>
+        <v>14835.59</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -5413,20 +5413,20 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>보령</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>9678.110000000001</v>
+        <v>16811.92</v>
       </c>
       <c r="D185" t="n">
-        <v>673.4</v>
+        <v>801.08</v>
       </c>
       <c r="E185" t="n">
-        <v>699.6799999999999</v>
+        <v>868.0700000000001</v>
       </c>
       <c r="F185" t="n">
-        <v>13738</v>
+        <v>17869.38</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -5440,20 +5440,20 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>코오롱인더</t>
+          <t>이수페타시스</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>33536.44</v>
+        <v>7187.29</v>
       </c>
       <c r="D186" t="n">
-        <v>669.42</v>
+        <v>784.8</v>
       </c>
       <c r="E186" t="n">
-        <v>116.17</v>
+        <v>652.48</v>
       </c>
       <c r="F186" t="n">
-        <v>56791.72</v>
+        <v>6871.52</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -5467,20 +5467,20 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>팜스코</t>
+          <t>현대홈쇼핑</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>14985.31</v>
+        <v>10898.89</v>
       </c>
       <c r="D187" t="n">
-        <v>664.6900000000001</v>
+        <v>773.33</v>
       </c>
       <c r="E187" t="n">
-        <v>-419.65</v>
+        <v>946.41</v>
       </c>
       <c r="F187" t="n">
-        <v>9116.49</v>
+        <v>18981.43</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -5494,20 +5494,20 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>한국토지신탁</t>
+          <t>녹십자</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2209.86</v>
+        <v>14603.54</v>
       </c>
       <c r="D188" t="n">
-        <v>663.15</v>
+        <v>765.24</v>
       </c>
       <c r="E188" t="n">
-        <v>279.22</v>
+        <v>485.4</v>
       </c>
       <c r="F188" t="n">
-        <v>16636.96</v>
+        <v>23917.58</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -5521,20 +5521,20 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>케이카</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>12053.2</v>
+        <v>24388.39</v>
       </c>
       <c r="D189" t="n">
-        <v>658.42</v>
+        <v>759.74</v>
       </c>
       <c r="E189" t="n">
-        <v>775.53</v>
+        <v>508.86</v>
       </c>
       <c r="F189" t="n">
-        <v>19787.4</v>
+        <v>5345.7</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -5548,20 +5548,20 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>SK오션플랜트</t>
+          <t>AJ네트웍스</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>9289.15</v>
+        <v>6982.77</v>
       </c>
       <c r="D190" t="n">
-        <v>656.87</v>
+        <v>750.92</v>
       </c>
       <c r="E190" t="n">
-        <v>377.9</v>
+        <v>286.31</v>
       </c>
       <c r="F190" t="n">
-        <v>10817.32</v>
+        <v>17031.29</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -5575,20 +5575,20 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>더블유게임즈</t>
+          <t>롯데정밀화학</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1773.38</v>
+        <v>17503.45</v>
       </c>
       <c r="D191" t="n">
-        <v>651.39</v>
+        <v>745.12</v>
       </c>
       <c r="E191" t="n">
-        <v>734.0700000000001</v>
+        <v>1030.29</v>
       </c>
       <c r="F191" t="n">
-        <v>7882.59</v>
+        <v>25389.86</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -5602,20 +5602,20 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>사조대림</t>
+          <t>현대코퍼레이션</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>14066.89</v>
+        <v>52558.5</v>
       </c>
       <c r="D192" t="n">
-        <v>650.5599999999999</v>
+        <v>732.89</v>
       </c>
       <c r="E192" t="n">
-        <v>424.22</v>
+        <v>864.4299999999999</v>
       </c>
       <c r="F192" t="n">
-        <v>10837.29</v>
+        <v>16802.64</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -5629,20 +5629,20 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>한화비전</t>
+          <t>빙그레</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>8216.040000000001</v>
+        <v>13124.34</v>
       </c>
       <c r="D193" t="n">
-        <v>631.26</v>
+        <v>730.79</v>
       </c>
       <c r="E193" t="n">
-        <v>-282.23</v>
+        <v>519.89</v>
       </c>
       <c r="F193" t="n">
-        <v>12336.68</v>
+        <v>10157.36</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -5656,20 +5656,20 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>달바글로벌</t>
+          <t>SNT홀딩스</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>3030.19</v>
+        <v>765.9</v>
       </c>
       <c r="D194" t="n">
-        <v>628.08</v>
+        <v>727.72</v>
       </c>
       <c r="E194" t="n">
-        <v>186.37</v>
+        <v>1374.78</v>
       </c>
       <c r="F194" t="n">
-        <v>1391.43</v>
+        <v>6049.49</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -5683,20 +5683,20 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>삼양홀딩스</t>
+          <t>덴티움</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2358.26</v>
+        <v>3207.23</v>
       </c>
       <c r="D195" t="n">
-        <v>618.4</v>
+        <v>706.26</v>
       </c>
       <c r="E195" t="n">
-        <v>740.75</v>
+        <v>267.33</v>
       </c>
       <c r="F195" t="n">
-        <v>26437.33</v>
+        <v>7373.13</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -5710,20 +5710,20 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>세아베스틸지주</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>5523.65</v>
+        <v>883.78</v>
       </c>
       <c r="D196" t="n">
-        <v>615.1799999999999</v>
+        <v>702.03</v>
       </c>
       <c r="E196" t="n">
-        <v>412.57</v>
+        <v>643.42</v>
       </c>
       <c r="F196" t="n">
-        <v>6892.79</v>
+        <v>18317.64</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -5737,20 +5737,20 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>해성디에스</t>
+          <t>LX홀딩스</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>5945.89</v>
+        <v>1041.2</v>
       </c>
       <c r="D197" t="n">
-        <v>609.52</v>
+        <v>701.53</v>
       </c>
       <c r="E197" t="n">
-        <v>555.15</v>
+        <v>757.67</v>
       </c>
       <c r="F197" t="n">
-        <v>7782.14</v>
+        <v>14084.78</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -5764,20 +5764,20 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>케이씨텍</t>
+          <t>HD현대마린엔진</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3833.92</v>
+        <v>3798.48</v>
       </c>
       <c r="D198" t="n">
-        <v>608.75</v>
+        <v>684.52</v>
       </c>
       <c r="E198" t="n">
-        <v>542.9400000000001</v>
+        <v>1573.79</v>
       </c>
       <c r="F198" t="n">
-        <v>6010.84</v>
+        <v>7833.44</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -5791,20 +5791,20 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>미원에스씨</t>
+          <t>TKG휴켐스</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>5060.03</v>
+        <v>10822.36</v>
       </c>
       <c r="D199" t="n">
-        <v>606.78</v>
+        <v>674.71</v>
       </c>
       <c r="E199" t="n">
-        <v>554.85</v>
+        <v>611.71</v>
       </c>
       <c r="F199" t="n">
-        <v>5195.47</v>
+        <v>10694.35</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -5818,20 +5818,20 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>삼천리</t>
+          <t>보령</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>36207.43</v>
+        <v>9678.110000000001</v>
       </c>
       <c r="D200" t="n">
-        <v>605.9</v>
+        <v>673.4</v>
       </c>
       <c r="E200" t="n">
-        <v>540.75</v>
+        <v>699.6799999999999</v>
       </c>
       <c r="F200" t="n">
-        <v>33439.31</v>
+        <v>13738</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -5845,20 +5845,20 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>동부건설</t>
+          <t>HL D&amp;I</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>16315.32</v>
+        <v>16451.9</v>
       </c>
       <c r="D201" t="n">
-        <v>604.87</v>
+        <v>672.03</v>
       </c>
       <c r="E201" t="n">
-        <v>460.02</v>
+        <v>244.39</v>
       </c>
       <c r="F201" t="n">
-        <v>15693.62</v>
+        <v>16806.03</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-03-22 23:25</t>
+          <t>2026-04-01 02:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Update KOSPI Top200 operating profit - 2026-07-01
</commit_message>
<xml_diff>
--- a/top200_operating_profit_kospi.xlsx
+++ b/top200_operating_profit_kospi.xlsx
@@ -580,20 +580,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>KB금융</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>787667.91</v>
+        <v>38923.51</v>
       </c>
       <c r="D6" t="n">
-        <v>35150.52</v>
+        <v>36591.14</v>
       </c>
       <c r="E6" t="n">
-        <v>40548.78</v>
+        <v>36576.33</v>
       </c>
       <c r="F6" t="n">
-        <v>985803.88</v>
+        <v>308531.4</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -607,20 +607,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>기업은행</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>273550.51</v>
+        <v>787667.91</v>
       </c>
       <c r="D7" t="n">
-        <v>32890.25</v>
+        <v>35150.52</v>
       </c>
       <c r="E7" t="n">
-        <v>24280.83</v>
+        <v>40548.78</v>
       </c>
       <c r="F7" t="n">
-        <v>4312784.52</v>
+        <v>985803.88</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -634,20 +634,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SK이노베이션</t>
+          <t>기업은행</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>48509.05</v>
+        <v>241586.59</v>
       </c>
       <c r="D8" t="n">
-        <v>27300.35</v>
+        <v>33217.8</v>
       </c>
       <c r="E8" t="n">
-        <v>27067.82</v>
+        <v>23858.46</v>
       </c>
       <c r="F8" t="n">
-        <v>397145.46</v>
+        <v>4571578.21</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -661,20 +661,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>SK이노베이션</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>219664.96</v>
+        <v>48509.05</v>
       </c>
       <c r="D9" t="n">
-        <v>26995.44</v>
+        <v>27300.35</v>
       </c>
       <c r="E9" t="n">
-        <v>20477.81</v>
+        <v>27067.82</v>
       </c>
       <c r="F9" t="n">
-        <v>852235.63</v>
+        <v>397145.46</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -688,20 +688,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DB손해보험</t>
+          <t>신한지주</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>188308.38</v>
+        <v>29569.74</v>
       </c>
       <c r="D10" t="n">
-        <v>23626.63</v>
+        <v>23643.16</v>
       </c>
       <c r="E10" t="n">
-        <v>17722.29</v>
+        <v>23854.57</v>
       </c>
       <c r="F10" t="n">
-        <v>528589.41</v>
+        <v>377938.27</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -715,20 +715,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KB금융</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>23768.33</v>
+        <v>239474.18</v>
       </c>
       <c r="D11" t="n">
-        <v>21706.45</v>
+        <v>23306.83</v>
       </c>
       <c r="E11" t="n">
-        <v>21705.97</v>
+        <v>16908.78</v>
       </c>
       <c r="F11" t="n">
-        <v>298068.23</v>
+        <v>938090.4399999999</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -742,20 +742,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>삼성바이오로직스</t>
+          <t>DB손해보험</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>45569.72</v>
+        <v>200210.58</v>
       </c>
       <c r="D12" t="n">
-        <v>20680.93</v>
+        <v>20877.8</v>
       </c>
       <c r="E12" t="n">
-        <v>15861.87</v>
+        <v>15348.8</v>
       </c>
       <c r="F12" t="n">
-        <v>110239.69</v>
+        <v>594088.28</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -769,20 +769,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HD현대중공업</t>
+          <t>삼성바이오로직스</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>175694.57</v>
+        <v>45569.72</v>
       </c>
       <c r="D13" t="n">
-        <v>20427.26</v>
+        <v>20680.93</v>
       </c>
       <c r="E13" t="n">
-        <v>14224.81</v>
+        <v>15861.87</v>
       </c>
       <c r="F13" t="n">
-        <v>261990.62</v>
+        <v>110239.69</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -796,20 +796,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>HD현대중공업</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>95251.38</v>
+        <v>175694.57</v>
       </c>
       <c r="D14" t="n">
-        <v>20226.04</v>
+        <v>20427.26</v>
       </c>
       <c r="E14" t="n">
-        <v>14675.05</v>
+        <v>14224.81</v>
       </c>
       <c r="F14" t="n">
-        <v>246513.33</v>
+        <v>261990.62</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -823,20 +823,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>70193.3</v>
+        <v>95251.38</v>
       </c>
       <c r="D15" t="n">
-        <v>19455.32</v>
+        <v>20226.04</v>
       </c>
       <c r="E15" t="n">
-        <v>18829.69</v>
+        <v>14675.05</v>
       </c>
       <c r="F15" t="n">
-        <v>203411.99</v>
+        <v>246513.33</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -850,20 +850,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>신한지주</t>
+          <t>NAVER</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>25565.03</v>
+        <v>70193.3</v>
       </c>
       <c r="D16" t="n">
-        <v>18008.63</v>
+        <v>19455.32</v>
       </c>
       <c r="E16" t="n">
-        <v>16198.67</v>
+        <v>18829.69</v>
       </c>
       <c r="F16" t="n">
-        <v>376723.03</v>
+        <v>203411.99</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -985,20 +985,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>한국금융지주</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>225317.96</v>
+        <v>18572.88</v>
       </c>
       <c r="D21" t="n">
-        <v>15612.98</v>
+        <v>16477.64</v>
       </c>
       <c r="E21" t="n">
-        <v>14605.15</v>
+        <v>16368.59</v>
       </c>
       <c r="F21" t="n">
-        <v>152215.75</v>
+        <v>139924.99</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1012,20 +1012,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>대한항공</t>
+          <t>현대글로비스</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>165018.52</v>
+        <v>225317.96</v>
       </c>
       <c r="D22" t="n">
-        <v>15392.52</v>
+        <v>15612.98</v>
       </c>
       <c r="E22" t="n">
-        <v>9649.299999999999</v>
+        <v>14605.15</v>
       </c>
       <c r="F22" t="n">
-        <v>384566.48</v>
+        <v>152215.75</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1039,20 +1039,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>대한항공</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>107211.77</v>
+        <v>165018.52</v>
       </c>
       <c r="D23" t="n">
-        <v>14232</v>
+        <v>15392.52</v>
       </c>
       <c r="E23" t="n">
-        <v>18512.82</v>
+        <v>9649.299999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>329632.63</v>
+        <v>384566.48</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1066,20 +1066,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>현대해상</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>172193.14</v>
+        <v>107211.77</v>
       </c>
       <c r="D24" t="n">
-        <v>14018.71</v>
+        <v>14232</v>
       </c>
       <c r="E24" t="n">
-        <v>10306.84</v>
+        <v>18512.82</v>
       </c>
       <c r="F24" t="n">
-        <v>479776.79</v>
+        <v>329632.63</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1093,20 +1093,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>키움증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>157151.87</v>
+        <v>145771.29</v>
       </c>
       <c r="D25" t="n">
-        <v>13254.58</v>
+        <v>13261.94</v>
       </c>
       <c r="E25" t="n">
-        <v>10994.04</v>
+        <v>9712.969999999999</v>
       </c>
       <c r="F25" t="n">
-        <v>688072.48</v>
+        <v>727563.24</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1120,20 +1120,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>키움증권</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>193240.24</v>
+        <v>157151.87</v>
       </c>
       <c r="D26" t="n">
-        <v>13049.73</v>
+        <v>13254.58</v>
       </c>
       <c r="E26" t="n">
-        <v>10617.53</v>
+        <v>10994.04</v>
       </c>
       <c r="F26" t="n">
-        <v>296775.87</v>
+        <v>688072.48</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1147,20 +1147,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>메리츠금융지주</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>13584.64</v>
+        <v>193240.24</v>
       </c>
       <c r="D27" t="n">
-        <v>12203.67</v>
+        <v>13049.73</v>
       </c>
       <c r="E27" t="n">
-        <v>12276.08</v>
+        <v>10617.53</v>
       </c>
       <c r="F27" t="n">
-        <v>52404.74</v>
+        <v>296775.87</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1174,20 +1174,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>고려아연</t>
+          <t>우리금융지주</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>105342.41</v>
+        <v>14786.54</v>
       </c>
       <c r="D28" t="n">
-        <v>11795.5</v>
+        <v>12947.15</v>
       </c>
       <c r="E28" t="n">
-        <v>7715.72</v>
+        <v>11270.4</v>
       </c>
       <c r="F28" t="n">
-        <v>169216.42</v>
+        <v>273943.72</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1201,20 +1201,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>129035.94</v>
+        <v>131888.21</v>
       </c>
       <c r="D29" t="n">
-        <v>11540.03</v>
+        <v>12742.17</v>
       </c>
       <c r="E29" t="n">
-        <v>13441.99</v>
+        <v>9083.01</v>
       </c>
       <c r="F29" t="n">
-        <v>197246.46</v>
+        <v>798198.4300000001</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1228,20 +1228,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>우리금융지주</t>
+          <t>메리츠금융지주</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>12625.33</v>
+        <v>14024.22</v>
       </c>
       <c r="D30" t="n">
-        <v>11233.01</v>
+        <v>12642.49</v>
       </c>
       <c r="E30" t="n">
-        <v>11233.32</v>
+        <v>12717.1</v>
       </c>
       <c r="F30" t="n">
-        <v>263530.37</v>
+        <v>53110.8</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1255,20 +1255,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>고려아연</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>129366.6</v>
+        <v>105342.41</v>
       </c>
       <c r="D31" t="n">
-        <v>11054.9</v>
+        <v>11795.5</v>
       </c>
       <c r="E31" t="n">
-        <v>8188.16</v>
+        <v>7715.72</v>
       </c>
       <c r="F31" t="n">
-        <v>569763.86</v>
+        <v>169216.42</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1282,20 +1282,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>크래프톤</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28856.5</v>
+        <v>129035.94</v>
       </c>
       <c r="D32" t="n">
-        <v>10627.18</v>
+        <v>11540.03</v>
       </c>
       <c r="E32" t="n">
-        <v>7351.51</v>
+        <v>13441.99</v>
       </c>
       <c r="F32" t="n">
-        <v>81595.94</v>
+        <v>197246.46</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1309,20 +1309,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>KT&amp;G</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>41454.75</v>
+        <v>212561.47</v>
       </c>
       <c r="D33" t="n">
-        <v>10007.17</v>
+        <v>11312.48</v>
       </c>
       <c r="E33" t="n">
-        <v>9198.23</v>
+        <v>5951.34</v>
       </c>
       <c r="F33" t="n">
-        <v>113642.92</v>
+        <v>1087875.47</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1336,20 +1336,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>크래프톤</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>56949.95</v>
+        <v>28856.5</v>
       </c>
       <c r="D34" t="n">
-        <v>9988.799999999999</v>
+        <v>10627.18</v>
       </c>
       <c r="E34" t="n">
-        <v>7433.49</v>
+        <v>7351.51</v>
       </c>
       <c r="F34" t="n">
-        <v>90510.12</v>
+        <v>81595.94</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1363,20 +1363,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>KT&amp;G</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>14033.1</v>
+        <v>41454.75</v>
       </c>
       <c r="D35" t="n">
-        <v>9768.25</v>
+        <v>10007.17</v>
       </c>
       <c r="E35" t="n">
-        <v>4948.78</v>
+        <v>9198.23</v>
       </c>
       <c r="F35" t="n">
-        <v>518155.85</v>
+        <v>113642.92</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1390,20 +1390,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>165863.46</v>
+        <v>56949.95</v>
       </c>
       <c r="D36" t="n">
-        <v>9241.860000000001</v>
+        <v>9988.799999999999</v>
       </c>
       <c r="E36" t="n">
-        <v>6991.3</v>
+        <v>7433.49</v>
       </c>
       <c r="F36" t="n">
-        <v>951663.41</v>
+        <v>90510.12</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1417,20 +1417,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>29286.38</v>
+        <v>14033.1</v>
       </c>
       <c r="D37" t="n">
-        <v>9189.52</v>
+        <v>9768.25</v>
       </c>
       <c r="E37" t="n">
-        <v>8475.43</v>
+        <v>4948.78</v>
       </c>
       <c r="F37" t="n">
-        <v>218130.1</v>
+        <v>518155.85</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1444,20 +1444,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>142042.31</v>
+        <v>29286.38</v>
       </c>
       <c r="D38" t="n">
-        <v>9117.41</v>
+        <v>9189.52</v>
       </c>
       <c r="E38" t="n">
-        <v>5427.99</v>
+        <v>8475.43</v>
       </c>
       <c r="F38" t="n">
-        <v>187145.25</v>
+        <v>218130.1</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1471,20 +1471,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HD현대일렉트릭</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>33811.39</v>
+        <v>142042.31</v>
       </c>
       <c r="D39" t="n">
-        <v>8891.57</v>
+        <v>9117.41</v>
       </c>
       <c r="E39" t="n">
-        <v>6364.38</v>
+        <v>5427.99</v>
       </c>
       <c r="F39" t="n">
-        <v>35038.24</v>
+        <v>187145.25</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1498,20 +1498,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>HD현대일렉트릭</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>94508.34</v>
+        <v>33811.39</v>
       </c>
       <c r="D40" t="n">
-        <v>8791.6</v>
+        <v>8891.57</v>
       </c>
       <c r="E40" t="n">
-        <v>6259.15</v>
+        <v>6364.38</v>
       </c>
       <c r="F40" t="n">
-        <v>592814.76</v>
+        <v>35038.24</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1660,20 +1660,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>현대해상</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>14937.54</v>
+        <v>175693.55</v>
       </c>
       <c r="D46" t="n">
-        <v>7006.49</v>
+        <v>7268.63</v>
       </c>
       <c r="E46" t="n">
-        <v>6143.35</v>
+        <v>5611.06</v>
       </c>
       <c r="F46" t="n">
-        <v>129011.26</v>
+        <v>496458.75</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1687,20 +1687,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>한국금융지주</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>7806.06</v>
+        <v>14937.54</v>
       </c>
       <c r="D47" t="n">
-        <v>6207.13</v>
+        <v>7006.49</v>
       </c>
       <c r="E47" t="n">
-        <v>6168.82</v>
+        <v>6143.35</v>
       </c>
       <c r="F47" t="n">
-        <v>109040.74</v>
+        <v>129011.26</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>29456.21</v>
+        <v>30862.91</v>
       </c>
       <c r="D48" t="n">
-        <v>6068.8</v>
+        <v>6493.71</v>
       </c>
       <c r="E48" t="n">
-        <v>4400.65</v>
+        <v>4802.8</v>
       </c>
       <c r="F48" t="n">
-        <v>628052.8199999999</v>
+        <v>764097.75</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1795,20 +1795,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>한화생명</t>
+          <t>BNK금융지주</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>133221.44</v>
+        <v>7061.9</v>
       </c>
       <c r="D51" t="n">
-        <v>5824.59</v>
+        <v>5832.03</v>
       </c>
       <c r="E51" t="n">
-        <v>7205.7</v>
+        <v>5827.62</v>
       </c>
       <c r="F51" t="n">
-        <v>1221350.33</v>
+        <v>72676.00999999999</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1876,20 +1876,20 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>삼성에스디에스</t>
+          <t>JB금융지주</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>54646.38</v>
+        <v>6033.67</v>
       </c>
       <c r="D54" t="n">
-        <v>5204.33</v>
+        <v>5252.89</v>
       </c>
       <c r="E54" t="n">
-        <v>4752.08</v>
+        <v>5265.74</v>
       </c>
       <c r="F54" t="n">
-        <v>84764.87</v>
+        <v>38119.64</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -1903,20 +1903,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>한화손해보험</t>
+          <t>F&amp;F</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>59675.46</v>
+        <v>16946.96</v>
       </c>
       <c r="D55" t="n">
-        <v>5033.89</v>
+        <v>5244.52</v>
       </c>
       <c r="E55" t="n">
-        <v>3822.76</v>
+        <v>3994.89</v>
       </c>
       <c r="F55" t="n">
-        <v>197526.8</v>
+        <v>22154.97</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -1930,20 +1930,20 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>삼성에스디에스</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>71170.23</v>
+        <v>54646.38</v>
       </c>
       <c r="D56" t="n">
-        <v>4960.06</v>
+        <v>5204.33</v>
       </c>
       <c r="E56" t="n">
-        <v>5076.66</v>
+        <v>4752.08</v>
       </c>
       <c r="F56" t="n">
-        <v>148663.75</v>
+        <v>84764.87</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -1957,20 +1957,20 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>41440.72</v>
+        <v>71170.23</v>
       </c>
       <c r="D57" t="n">
-        <v>4850.72</v>
+        <v>4960.06</v>
       </c>
       <c r="E57" t="n">
-        <v>2983.47</v>
+        <v>5076.66</v>
       </c>
       <c r="F57" t="n">
-        <v>107163.79</v>
+        <v>148663.75</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -1984,20 +1984,20 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>GS건설</t>
+          <t>한화손해보험</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>81002.07000000001</v>
+        <v>69795.77</v>
       </c>
       <c r="D58" t="n">
-        <v>4811.25</v>
+        <v>4884.62</v>
       </c>
       <c r="E58" t="n">
-        <v>399.67</v>
+        <v>3610.59</v>
       </c>
       <c r="F58" t="n">
-        <v>131632.9</v>
+        <v>202790.52</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2011,20 +2011,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>팬오션</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>19018.34</v>
+        <v>41440.72</v>
       </c>
       <c r="D59" t="n">
-        <v>4713.97</v>
+        <v>4850.72</v>
       </c>
       <c r="E59" t="n">
-        <v>3553.03</v>
+        <v>2983.47</v>
       </c>
       <c r="F59" t="n">
-        <v>18927.11</v>
+        <v>107163.79</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2038,20 +2038,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>GS건설</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>40978.14</v>
+        <v>81002.07000000001</v>
       </c>
       <c r="D60" t="n">
-        <v>4423.78</v>
+        <v>4811.25</v>
       </c>
       <c r="E60" t="n">
-        <v>2745.11</v>
+        <v>399.67</v>
       </c>
       <c r="F60" t="n">
-        <v>51014.56</v>
+        <v>131632.9</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2065,20 +2065,20 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>26808.61</v>
+        <v>19018.34</v>
       </c>
       <c r="D61" t="n">
-        <v>4402.42</v>
+        <v>4713.97</v>
       </c>
       <c r="E61" t="n">
-        <v>2341.92</v>
+        <v>3553.03</v>
       </c>
       <c r="F61" t="n">
-        <v>115903.69</v>
+        <v>18927.11</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2092,20 +2092,20 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HD현대</t>
+          <t>코리안리</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5260.74</v>
+        <v>65760.88</v>
       </c>
       <c r="D62" t="n">
-        <v>4391.82</v>
+        <v>4633.31</v>
       </c>
       <c r="E62" t="n">
-        <v>4020.47</v>
+        <v>3165.81</v>
       </c>
       <c r="F62" t="n">
-        <v>89930.52</v>
+        <v>139998.05</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2119,20 +2119,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>JB금융지주</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>5052.56</v>
+        <v>40978.14</v>
       </c>
       <c r="D63" t="n">
-        <v>4336.51</v>
+        <v>4423.78</v>
       </c>
       <c r="E63" t="n">
-        <v>4336.22</v>
+        <v>2745.11</v>
       </c>
       <c r="F63" t="n">
-        <v>34207.97</v>
+        <v>51014.56</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2146,20 +2146,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>LG씨엔에스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>54492.71</v>
+        <v>26808.61</v>
       </c>
       <c r="D64" t="n">
-        <v>4335.34</v>
+        <v>4402.42</v>
       </c>
       <c r="E64" t="n">
-        <v>3888.54</v>
+        <v>2341.92</v>
       </c>
       <c r="F64" t="n">
-        <v>48322.18</v>
+        <v>115903.69</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2173,20 +2173,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>롯데쇼핑</t>
+          <t>HD현대</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>81880.61</v>
+        <v>5260.74</v>
       </c>
       <c r="D65" t="n">
-        <v>4112.35</v>
+        <v>4391.82</v>
       </c>
       <c r="E65" t="n">
-        <v>1104.16</v>
+        <v>4020.47</v>
       </c>
       <c r="F65" t="n">
-        <v>303486.58</v>
+        <v>89930.52</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2200,20 +2200,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>금호타이어</t>
+          <t>LG씨엔에스</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>35308.91</v>
+        <v>54492.71</v>
       </c>
       <c r="D66" t="n">
-        <v>4082.13</v>
+        <v>4335.34</v>
       </c>
       <c r="E66" t="n">
-        <v>3829.93</v>
+        <v>3888.54</v>
       </c>
       <c r="F66" t="n">
-        <v>39988.07</v>
+        <v>48322.18</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2227,20 +2227,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>F&amp;F</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>15179.94</v>
+        <v>44605.17</v>
       </c>
       <c r="D67" t="n">
-        <v>4024.07</v>
+        <v>4155.24</v>
       </c>
       <c r="E67" t="n">
-        <v>3235.32</v>
+        <v>4741.01</v>
       </c>
       <c r="F67" t="n">
-        <v>19235.04</v>
+        <v>287972.24</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2254,20 +2254,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>롯데쇼핑</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>215960.08</v>
+        <v>81880.61</v>
       </c>
       <c r="D68" t="n">
-        <v>4007.06</v>
+        <v>4112.35</v>
       </c>
       <c r="E68" t="n">
-        <v>2592.17</v>
+        <v>1104.16</v>
       </c>
       <c r="F68" t="n">
-        <v>101904.14</v>
+        <v>303486.58</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2281,20 +2281,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>코리안리</t>
+          <t>금호타이어</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>68031.78</v>
+        <v>35308.91</v>
       </c>
       <c r="D69" t="n">
-        <v>3994.96</v>
+        <v>4082.13</v>
       </c>
       <c r="E69" t="n">
-        <v>2858.73</v>
+        <v>3829.93</v>
       </c>
       <c r="F69" t="n">
-        <v>129267.22</v>
+        <v>39988.07</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2308,20 +2308,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>두산밥캣</t>
+          <t>한화생명</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4903.43</v>
+        <v>144741.87</v>
       </c>
       <c r="D70" t="n">
-        <v>3935.42</v>
+        <v>4014.37</v>
       </c>
       <c r="E70" t="n">
-        <v>3690.68</v>
+        <v>3133.2</v>
       </c>
       <c r="F70" t="n">
-        <v>40606.56</v>
+        <v>1257765.82</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2335,20 +2335,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>동양생명</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>34667.35</v>
+        <v>215960.08</v>
       </c>
       <c r="D71" t="n">
-        <v>3790.53</v>
+        <v>4007.06</v>
       </c>
       <c r="E71" t="n">
-        <v>3101.58</v>
+        <v>2592.17</v>
       </c>
       <c r="F71" t="n">
-        <v>345775.75</v>
+        <v>101904.14</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2362,20 +2362,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LIG넥스원</t>
+          <t>두산밥캣</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>42899.85</v>
+        <v>4903.43</v>
       </c>
       <c r="D72" t="n">
-        <v>3645.2</v>
+        <v>3935.42</v>
       </c>
       <c r="E72" t="n">
-        <v>2534.49</v>
+        <v>3690.68</v>
       </c>
       <c r="F72" t="n">
-        <v>78329.21000000001</v>
+        <v>40606.56</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2389,20 +2389,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LS ELECTRIC</t>
+          <t>서울보증보험</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>34627.41</v>
+        <v>27352.7</v>
       </c>
       <c r="D73" t="n">
-        <v>3621.94</v>
+        <v>3713.3</v>
       </c>
       <c r="E73" t="n">
-        <v>2938.25</v>
+        <v>2642.44</v>
       </c>
       <c r="F73" t="n">
-        <v>39999.49</v>
+        <v>93738.28999999999</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2416,20 +2416,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>LIG디펜스앤에어로스페이스</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>83779.08</v>
+        <v>42899.85</v>
       </c>
       <c r="D74" t="n">
-        <v>3559.4</v>
+        <v>3645.2</v>
       </c>
       <c r="E74" t="n">
-        <v>3918.63</v>
+        <v>2534.49</v>
       </c>
       <c r="F74" t="n">
-        <v>100939.74</v>
+        <v>78329.21000000001</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2443,20 +2443,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LS ELECTRIC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>15282.96</v>
+        <v>34627.41</v>
       </c>
       <c r="D75" t="n">
-        <v>3541.22</v>
+        <v>3621.94</v>
       </c>
       <c r="E75" t="n">
-        <v>2899.39</v>
+        <v>2938.25</v>
       </c>
       <c r="F75" t="n">
-        <v>7342.98</v>
+        <v>39999.49</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2470,20 +2470,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CJ대한통운</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>83538.53</v>
+        <v>83779.08</v>
       </c>
       <c r="D76" t="n">
-        <v>3531.28</v>
+        <v>3559.4</v>
       </c>
       <c r="E76" t="n">
-        <v>2069.36</v>
+        <v>3918.63</v>
       </c>
       <c r="F76" t="n">
-        <v>80788.06</v>
+        <v>100939.74</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2497,20 +2497,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>46879.55</v>
+        <v>15282.96</v>
       </c>
       <c r="D77" t="n">
-        <v>3426.07</v>
+        <v>3541.22</v>
       </c>
       <c r="E77" t="n">
-        <v>3916.85</v>
+        <v>2899.39</v>
       </c>
       <c r="F77" t="n">
-        <v>76021.44</v>
+        <v>7342.98</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2524,20 +2524,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>CJ대한통운</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>43152.04</v>
+        <v>83538.53</v>
       </c>
       <c r="D78" t="n">
-        <v>3414.97</v>
+        <v>3531.28</v>
       </c>
       <c r="E78" t="n">
-        <v>488.1</v>
+        <v>2069.36</v>
       </c>
       <c r="F78" t="n">
-        <v>112011.1</v>
+        <v>80788.06</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2551,20 +2551,20 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>HD현대마린솔루션</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>14745.03</v>
+        <v>46879.55</v>
       </c>
       <c r="D79" t="n">
-        <v>3306.95</v>
+        <v>3426.07</v>
       </c>
       <c r="E79" t="n">
-        <v>2552.42</v>
+        <v>3916.85</v>
       </c>
       <c r="F79" t="n">
-        <v>11180.68</v>
+        <v>76021.44</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2578,20 +2578,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>17675.96</v>
+        <v>43152.04</v>
       </c>
       <c r="D80" t="n">
-        <v>3282.01</v>
+        <v>3414.97</v>
       </c>
       <c r="E80" t="n">
-        <v>2806.19</v>
+        <v>488.1</v>
       </c>
       <c r="F80" t="n">
-        <v>67539.56</v>
+        <v>112011.1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2605,20 +2605,20 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>HD현대마린솔루션</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3978.62</v>
+        <v>14745.03</v>
       </c>
       <c r="D81" t="n">
-        <v>3150.08</v>
+        <v>3306.95</v>
       </c>
       <c r="E81" t="n">
-        <v>2755.98</v>
+        <v>2552.42</v>
       </c>
       <c r="F81" t="n">
-        <v>59512.09</v>
+        <v>11180.68</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -2632,20 +2632,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>미스토홀딩스</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3434.28</v>
+        <v>17675.96</v>
       </c>
       <c r="D82" t="n">
-        <v>3107.36</v>
+        <v>3282.01</v>
       </c>
       <c r="E82" t="n">
-        <v>3120.43</v>
+        <v>2806.19</v>
       </c>
       <c r="F82" t="n">
-        <v>7944.7</v>
+        <v>67539.56</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -2659,20 +2659,20 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>12137.76</v>
+        <v>3978.62</v>
       </c>
       <c r="D83" t="n">
-        <v>3019.39</v>
+        <v>3150.08</v>
       </c>
       <c r="E83" t="n">
-        <v>2718.1</v>
+        <v>2755.98</v>
       </c>
       <c r="F83" t="n">
-        <v>25142.22</v>
+        <v>59512.09</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -2686,20 +2686,20 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>미스토홀딩스</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3575.72</v>
+        <v>3434.28</v>
       </c>
       <c r="D84" t="n">
-        <v>3006.52</v>
+        <v>3107.36</v>
       </c>
       <c r="E84" t="n">
-        <v>-1055.72</v>
+        <v>3120.43</v>
       </c>
       <c r="F84" t="n">
-        <v>65984.14</v>
+        <v>7944.7</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -2713,20 +2713,20 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>GS리테일</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>117746.44</v>
+        <v>12137.76</v>
       </c>
       <c r="D85" t="n">
-        <v>2898.97</v>
+        <v>3019.39</v>
       </c>
       <c r="E85" t="n">
-        <v>841.17</v>
+        <v>2718.1</v>
       </c>
       <c r="F85" t="n">
-        <v>71213.37</v>
+        <v>25142.22</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -2740,20 +2740,20 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>롯데렌탈</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>26738.1</v>
+        <v>3575.72</v>
       </c>
       <c r="D86" t="n">
-        <v>2874.97</v>
+        <v>3006.52</v>
       </c>
       <c r="E86" t="n">
-        <v>1070.42</v>
+        <v>-1055.72</v>
       </c>
       <c r="F86" t="n">
-        <v>66832.8</v>
+        <v>65984.14</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -2767,20 +2767,20 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>KCC</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>29357.24</v>
+        <v>12274.04</v>
       </c>
       <c r="D87" t="n">
-        <v>2828.34</v>
+        <v>2942.12</v>
       </c>
       <c r="E87" t="n">
-        <v>20648.95</v>
+        <v>2488.65</v>
       </c>
       <c r="F87" t="n">
-        <v>151265.49</v>
+        <v>15372.9</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -2794,20 +2794,20 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>GS</t>
+          <t>GS리테일</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3692.7</v>
+        <v>117746.44</v>
       </c>
       <c r="D88" t="n">
-        <v>2816.1</v>
+        <v>2898.97</v>
       </c>
       <c r="E88" t="n">
-        <v>2499.03</v>
+        <v>841.17</v>
       </c>
       <c r="F88" t="n">
-        <v>68684.23</v>
+        <v>71213.37</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -2821,20 +2821,20 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>롯데렌탈</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>30914.85</v>
+        <v>26738.1</v>
       </c>
       <c r="D89" t="n">
-        <v>2799.78</v>
+        <v>2874.97</v>
       </c>
       <c r="E89" t="n">
-        <v>3670.39</v>
+        <v>1070.42</v>
       </c>
       <c r="F89" t="n">
-        <v>93434.23</v>
+        <v>66832.8</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -2848,20 +2848,20 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>이마트</t>
+          <t>KCC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>166288.56</v>
+        <v>29357.24</v>
       </c>
       <c r="D90" t="n">
-        <v>2770.72</v>
+        <v>2828.34</v>
       </c>
       <c r="E90" t="n">
-        <v>520.0599999999999</v>
+        <v>20648.95</v>
       </c>
       <c r="F90" t="n">
-        <v>207466.93</v>
+        <v>151265.49</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -2875,20 +2875,20 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>서울보증보험</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>27246.02</v>
+        <v>3692.7</v>
       </c>
       <c r="D91" t="n">
-        <v>2744.37</v>
+        <v>2816.1</v>
       </c>
       <c r="E91" t="n">
-        <v>2109.55</v>
+        <v>2499.03</v>
       </c>
       <c r="F91" t="n">
-        <v>93029.48</v>
+        <v>68684.23</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -2902,20 +2902,20 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>영원무역</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>25074.15</v>
+        <v>30914.85</v>
       </c>
       <c r="D92" t="n">
-        <v>2727.61</v>
+        <v>2799.78</v>
       </c>
       <c r="E92" t="n">
-        <v>2636.21</v>
+        <v>3670.39</v>
       </c>
       <c r="F92" t="n">
-        <v>25812.27</v>
+        <v>93434.23</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -2929,20 +2929,20 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>효성</t>
+          <t>이마트</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>5523.08</v>
+        <v>166288.56</v>
       </c>
       <c r="D93" t="n">
-        <v>2703.63</v>
+        <v>2770.72</v>
       </c>
       <c r="E93" t="n">
-        <v>3306.05</v>
+        <v>520.0599999999999</v>
       </c>
       <c r="F93" t="n">
-        <v>33037.02</v>
+        <v>207466.93</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -2956,20 +2956,20 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>영원무역</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>36252.39</v>
+        <v>25074.15</v>
       </c>
       <c r="D94" t="n">
-        <v>2683.22</v>
+        <v>2727.61</v>
       </c>
       <c r="E94" t="n">
-        <v>1926.99</v>
+        <v>2636.21</v>
       </c>
       <c r="F94" t="n">
-        <v>101972.74</v>
+        <v>25812.27</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -2983,20 +2983,20 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>BNK금융지주</t>
+          <t>효성</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3770.69</v>
+        <v>5523.08</v>
       </c>
       <c r="D95" t="n">
-        <v>2658.58</v>
+        <v>2703.63</v>
       </c>
       <c r="E95" t="n">
-        <v>2656.02</v>
+        <v>3306.05</v>
       </c>
       <c r="F95" t="n">
-        <v>70504.62</v>
+        <v>33037.02</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3010,20 +3010,20 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>현대백화점</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>17955.45</v>
+        <v>36252.39</v>
       </c>
       <c r="D96" t="n">
-        <v>2647.55</v>
+        <v>2683.22</v>
       </c>
       <c r="E96" t="n">
-        <v>1416.93</v>
+        <v>1926.99</v>
       </c>
       <c r="F96" t="n">
-        <v>77964.71000000001</v>
+        <v>101972.74</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -3037,20 +3037,20 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SK가스</t>
+          <t>현대백화점</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>40564.98</v>
+        <v>17955.45</v>
       </c>
       <c r="D97" t="n">
-        <v>2617.72</v>
+        <v>2647.55</v>
       </c>
       <c r="E97" t="n">
-        <v>1427.91</v>
+        <v>1416.93</v>
       </c>
       <c r="F97" t="n">
-        <v>56380.69</v>
+        <v>77964.71000000001</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3064,20 +3064,20 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>iM금융지주</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>165124.62</v>
+        <v>3669.66</v>
       </c>
       <c r="D98" t="n">
-        <v>2511.83</v>
+        <v>2633.73</v>
       </c>
       <c r="E98" t="n">
-        <v>2313.3</v>
+        <v>2477.8</v>
       </c>
       <c r="F98" t="n">
-        <v>171912.83</v>
+        <v>51581.05</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3091,20 +3091,20 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>풍산</t>
+          <t>SK가스</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>38491.07</v>
+        <v>40564.98</v>
       </c>
       <c r="D99" t="n">
-        <v>2471.54</v>
+        <v>2617.72</v>
       </c>
       <c r="E99" t="n">
-        <v>1474.06</v>
+        <v>1427.91</v>
       </c>
       <c r="F99" t="n">
-        <v>38473.95</v>
+        <v>56380.69</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -3118,20 +3118,20 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HDC현대산업개발</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>40892.93</v>
+        <v>165124.62</v>
       </c>
       <c r="D100" t="n">
-        <v>2459.92</v>
+        <v>2511.83</v>
       </c>
       <c r="E100" t="n">
-        <v>1647.83</v>
+        <v>2313.3</v>
       </c>
       <c r="F100" t="n">
-        <v>72542.24000000001</v>
+        <v>171912.83</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -3145,20 +3145,20 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SK바이오팜</t>
+          <t>풍산</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>6506.12</v>
+        <v>38491.07</v>
       </c>
       <c r="D101" t="n">
-        <v>2455.79</v>
+        <v>2471.54</v>
       </c>
       <c r="E101" t="n">
-        <v>2482.68</v>
+        <v>1474.06</v>
       </c>
       <c r="F101" t="n">
-        <v>9554.690000000001</v>
+        <v>38473.95</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -3172,20 +3172,20 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>IPARK현대산업개발</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>5596.8</v>
+        <v>40892.93</v>
       </c>
       <c r="D102" t="n">
-        <v>2423.64</v>
+        <v>2459.92</v>
       </c>
       <c r="E102" t="n">
-        <v>2082.76</v>
+        <v>1647.83</v>
       </c>
       <c r="F102" t="n">
-        <v>7986.23</v>
+        <v>72542.24000000001</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -3199,20 +3199,20 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>신세계</t>
+          <t>SK바이오팜</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>20025.53</v>
+        <v>6506.12</v>
       </c>
       <c r="D103" t="n">
-        <v>2387.6</v>
+        <v>2455.79</v>
       </c>
       <c r="E103" t="n">
-        <v>595.25</v>
+        <v>2482.68</v>
       </c>
       <c r="F103" t="n">
-        <v>93785.89</v>
+        <v>9554.690000000001</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -3226,20 +3226,20 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>강원랜드</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>14753.61</v>
+        <v>5596.8</v>
       </c>
       <c r="D104" t="n">
-        <v>2354.71</v>
+        <v>2423.64</v>
       </c>
       <c r="E104" t="n">
-        <v>3072.46</v>
+        <v>2082.76</v>
       </c>
       <c r="F104" t="n">
-        <v>48199.87</v>
+        <v>7986.23</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -3253,20 +3253,20 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>S-Oil</t>
+          <t>신세계</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>338960.41</v>
+        <v>20025.53</v>
       </c>
       <c r="D105" t="n">
-        <v>2309.03</v>
+        <v>2387.6</v>
       </c>
       <c r="E105" t="n">
-        <v>1869.07</v>
+        <v>595.25</v>
       </c>
       <c r="F105" t="n">
-        <v>265200.56</v>
+        <v>93785.89</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -3280,20 +3280,20 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>강원랜드</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>47501.15</v>
+        <v>14753.61</v>
       </c>
       <c r="D106" t="n">
-        <v>2293.18</v>
+        <v>2354.71</v>
       </c>
       <c r="E106" t="n">
-        <v>977.03</v>
+        <v>3072.46</v>
       </c>
       <c r="F106" t="n">
-        <v>68784.28999999999</v>
+        <v>48199.87</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -3307,20 +3307,20 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>에스원</t>
+          <t>S-Oil</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>28596.77</v>
+        <v>338960.41</v>
       </c>
       <c r="D107" t="n">
-        <v>2274.64</v>
+        <v>2309.03</v>
       </c>
       <c r="E107" t="n">
-        <v>1905.62</v>
+        <v>1869.07</v>
       </c>
       <c r="F107" t="n">
-        <v>23402.37</v>
+        <v>265200.56</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -3334,20 +3334,20 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>71141.53999999999</v>
+        <v>47501.15</v>
       </c>
       <c r="D108" t="n">
-        <v>2260.22</v>
+        <v>2293.18</v>
       </c>
       <c r="E108" t="n">
-        <v>1078.99</v>
+        <v>977.03</v>
       </c>
       <c r="F108" t="n">
-        <v>40876.36</v>
+        <v>68784.28999999999</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -3361,20 +3361,20 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>BGF리테일</t>
+          <t>에스원</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>88581.22</v>
+        <v>28596.77</v>
       </c>
       <c r="D109" t="n">
-        <v>2219.57</v>
+        <v>2274.64</v>
       </c>
       <c r="E109" t="n">
-        <v>1740.74</v>
+        <v>1905.62</v>
       </c>
       <c r="F109" t="n">
-        <v>34209.89</v>
+        <v>23402.37</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -3388,20 +3388,20 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>아모레퍼시픽</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>26537.26</v>
+        <v>71141.53999999999</v>
       </c>
       <c r="D110" t="n">
-        <v>2125.15</v>
+        <v>2260.22</v>
       </c>
       <c r="E110" t="n">
-        <v>3179.2</v>
+        <v>1078.99</v>
       </c>
       <c r="F110" t="n">
-        <v>56252.44</v>
+        <v>40876.36</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -3415,20 +3415,20 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>에스엘</t>
+          <t>BGF리테일</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>29690.29</v>
+        <v>88581.22</v>
       </c>
       <c r="D111" t="n">
-        <v>2073.32</v>
+        <v>2219.57</v>
       </c>
       <c r="E111" t="n">
-        <v>2069.5</v>
+        <v>1740.74</v>
       </c>
       <c r="F111" t="n">
-        <v>26146.19</v>
+        <v>34209.89</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -3442,20 +3442,20 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>13909.95</v>
+        <v>32500.41</v>
       </c>
       <c r="D112" t="n">
-        <v>2035.63</v>
+        <v>2155.95</v>
       </c>
       <c r="E112" t="n">
-        <v>1662.56</v>
+        <v>1606.56</v>
       </c>
       <c r="F112" t="n">
-        <v>21009.97</v>
+        <v>31007.97</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -3469,20 +3469,20 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>한국앤컴퍼니</t>
+          <t>아모레퍼시픽</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>11007.84</v>
+        <v>26537.26</v>
       </c>
       <c r="D113" t="n">
-        <v>2015.15</v>
+        <v>2125.15</v>
       </c>
       <c r="E113" t="n">
-        <v>1587.63</v>
+        <v>3179.2</v>
       </c>
       <c r="F113" t="n">
-        <v>29550.88</v>
+        <v>56252.44</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -3496,20 +3496,20 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>금호석유화학</t>
+          <t>에스엘</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>45719.79</v>
+        <v>29690.29</v>
       </c>
       <c r="D114" t="n">
-        <v>1981.21</v>
+        <v>2073.32</v>
       </c>
       <c r="E114" t="n">
-        <v>1757.31</v>
+        <v>2069.5</v>
       </c>
       <c r="F114" t="n">
-        <v>46201.49</v>
+        <v>26146.19</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -3523,20 +3523,20 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>현대오토에버</t>
+          <t>동양생명</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>29434.44</v>
+        <v>35382.48</v>
       </c>
       <c r="D115" t="n">
-        <v>1968.51</v>
+        <v>2049.35</v>
       </c>
       <c r="E115" t="n">
-        <v>1626.95</v>
+        <v>658.37</v>
       </c>
       <c r="F115" t="n">
-        <v>29791.66</v>
+        <v>353152.58</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -3550,20 +3550,20 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>오리온</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>11458.38</v>
+        <v>13909.95</v>
       </c>
       <c r="D116" t="n">
-        <v>1868.17</v>
+        <v>2035.63</v>
       </c>
       <c r="E116" t="n">
-        <v>4003.12</v>
+        <v>1662.56</v>
       </c>
       <c r="F116" t="n">
-        <v>19453.14</v>
+        <v>21009.97</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -3577,20 +3577,20 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>CJ제일제당</t>
+          <t>한국앤컴퍼니</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>72811.41</v>
+        <v>11007.84</v>
       </c>
       <c r="D117" t="n">
-        <v>1856.31</v>
+        <v>2015.15</v>
       </c>
       <c r="E117" t="n">
-        <v>-5896.05</v>
+        <v>1587.63</v>
       </c>
       <c r="F117" t="n">
-        <v>106127.75</v>
+        <v>29550.88</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -3604,20 +3604,20 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>대한해운</t>
+          <t>금호석유화학</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>8566.25</v>
+        <v>45719.79</v>
       </c>
       <c r="D118" t="n">
-        <v>1814.1</v>
+        <v>1981.21</v>
       </c>
       <c r="E118" t="n">
-        <v>1486.71</v>
+        <v>1757.31</v>
       </c>
       <c r="F118" t="n">
-        <v>22826.67</v>
+        <v>46201.49</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -3631,20 +3631,20 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>산일전기</t>
+          <t>흥국화재</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>5019.46</v>
+        <v>35328.42</v>
       </c>
       <c r="D119" t="n">
-        <v>1790.4</v>
+        <v>1875.04</v>
       </c>
       <c r="E119" t="n">
-        <v>1491.41</v>
+        <v>1516.89</v>
       </c>
       <c r="F119" t="n">
-        <v>6811.01</v>
+        <v>125021.41</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -3658,20 +3658,20 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>하이트진로</t>
+          <t>오리온</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>22404.32</v>
+        <v>11458.38</v>
       </c>
       <c r="D120" t="n">
-        <v>1723.46</v>
+        <v>1868.17</v>
       </c>
       <c r="E120" t="n">
-        <v>480.04</v>
+        <v>4003.12</v>
       </c>
       <c r="F120" t="n">
-        <v>30334.13</v>
+        <v>19453.14</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -3685,20 +3685,20 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>교보증권</t>
+          <t>미래에셋생명</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>31683.52</v>
+        <v>50513.97</v>
       </c>
       <c r="D121" t="n">
-        <v>1677.37</v>
+        <v>1858.56</v>
       </c>
       <c r="E121" t="n">
-        <v>1371.03</v>
+        <v>1249</v>
       </c>
       <c r="F121" t="n">
-        <v>152533.09</v>
+        <v>328551.82</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -3712,20 +3712,20 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>현대위아</t>
+          <t>CJ제일제당</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>72787.97</v>
+        <v>72811.41</v>
       </c>
       <c r="D122" t="n">
-        <v>1676.1</v>
+        <v>1856.31</v>
       </c>
       <c r="E122" t="n">
-        <v>-184.68</v>
+        <v>-5896.05</v>
       </c>
       <c r="F122" t="n">
-        <v>55756.53</v>
+        <v>106127.75</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -3739,20 +3739,20 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>아이에스동서</t>
+          <t>시프트업</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>9514.799999999999</v>
+        <v>2945.46</v>
       </c>
       <c r="D123" t="n">
-        <v>1660.74</v>
+        <v>1814.18</v>
       </c>
       <c r="E123" t="n">
-        <v>-1623.32</v>
+        <v>1810.24</v>
       </c>
       <c r="F123" t="n">
-        <v>29895.06</v>
+        <v>10712.56</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -3766,20 +3766,20 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>한국타이어앤테크놀로지</t>
+          <t>교보증권</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>36484.38</v>
+        <v>44641.82</v>
       </c>
       <c r="D124" t="n">
-        <v>1624.95</v>
+        <v>1802.12</v>
       </c>
       <c r="E124" t="n">
-        <v>9907.75</v>
+        <v>1392.68</v>
       </c>
       <c r="F124" t="n">
-        <v>88571.17</v>
+        <v>185720.88</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -3793,20 +3793,20 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>산일전기</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1745.8</v>
+        <v>5019.46</v>
       </c>
       <c r="D125" t="n">
-        <v>1605.6</v>
+        <v>1790.4</v>
       </c>
       <c r="E125" t="n">
-        <v>1905.17</v>
+        <v>1491.41</v>
       </c>
       <c r="F125" t="n">
-        <v>38519.64</v>
+        <v>6811.01</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -3820,20 +3820,20 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>10746.19</v>
+        <v>11466.22</v>
       </c>
       <c r="D126" t="n">
-        <v>1581.86</v>
+        <v>1778.03</v>
       </c>
       <c r="E126" t="n">
-        <v>1722.95</v>
+        <v>1279.78</v>
       </c>
       <c r="F126" t="n">
-        <v>13490.33</v>
+        <v>14646.59</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -3847,20 +3847,20 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>동원산업</t>
+          <t>하이트진로</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>11062.5</v>
+        <v>22404.32</v>
       </c>
       <c r="D127" t="n">
-        <v>1556.56</v>
+        <v>1723.46</v>
       </c>
       <c r="E127" t="n">
-        <v>1278.59</v>
+        <v>480.04</v>
       </c>
       <c r="F127" t="n">
-        <v>36130.59</v>
+        <v>30334.13</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -3874,20 +3874,20 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>코스맥스</t>
+          <t>현대위아</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>15264.15</v>
+        <v>72787.97</v>
       </c>
       <c r="D128" t="n">
-        <v>1545.78</v>
+        <v>1676.1</v>
       </c>
       <c r="E128" t="n">
-        <v>1311.61</v>
+        <v>-184.68</v>
       </c>
       <c r="F128" t="n">
-        <v>13649.39</v>
+        <v>55756.53</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -3901,20 +3901,20 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>한국타이어앤테크놀로지</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>20182.27</v>
+        <v>36484.38</v>
       </c>
       <c r="D129" t="n">
-        <v>1535.19</v>
+        <v>1624.95</v>
       </c>
       <c r="E129" t="n">
-        <v>1065.76</v>
+        <v>9907.75</v>
       </c>
       <c r="F129" t="n">
-        <v>14784.9</v>
+        <v>88571.17</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -3928,20 +3928,20 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>시프트업</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2240.85</v>
+        <v>1745.8</v>
       </c>
       <c r="D130" t="n">
-        <v>1526.76</v>
+        <v>1605.6</v>
       </c>
       <c r="E130" t="n">
-        <v>1479.73</v>
+        <v>1905.17</v>
       </c>
       <c r="F130" t="n">
-        <v>8038.32</v>
+        <v>38519.64</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -3955,20 +3955,20 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>계룡건설</t>
+          <t>동원산업</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>20235.46</v>
+        <v>11062.5</v>
       </c>
       <c r="D131" t="n">
-        <v>1525.02</v>
+        <v>1556.56</v>
       </c>
       <c r="E131" t="n">
-        <v>1132.15</v>
+        <v>1278.59</v>
       </c>
       <c r="F131" t="n">
-        <v>22872.78</v>
+        <v>36130.59</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -3982,20 +3982,20 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>현대엘리베이터</t>
+          <t>코스맥스</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>16071</v>
+        <v>15264.15</v>
       </c>
       <c r="D132" t="n">
-        <v>1508.32</v>
+        <v>1545.78</v>
       </c>
       <c r="E132" t="n">
-        <v>3111.36</v>
+        <v>1311.61</v>
       </c>
       <c r="F132" t="n">
-        <v>27628.05</v>
+        <v>13649.39</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -4009,20 +4009,20 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>대상</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>35288.56</v>
+        <v>20182.27</v>
       </c>
       <c r="D133" t="n">
-        <v>1505.19</v>
+        <v>1535.19</v>
       </c>
       <c r="E133" t="n">
-        <v>-2855.56</v>
+        <v>1065.76</v>
       </c>
       <c r="F133" t="n">
-        <v>30613.98</v>
+        <v>14784.9</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -4036,20 +4036,20 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>계룡건설</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>11927.52</v>
+        <v>20235.46</v>
       </c>
       <c r="D134" t="n">
-        <v>1495.33</v>
+        <v>1525.02</v>
       </c>
       <c r="E134" t="n">
-        <v>1142.71</v>
+        <v>1132.15</v>
       </c>
       <c r="F134" t="n">
-        <v>15290.03</v>
+        <v>22872.78</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -4063,20 +4063,20 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>흥국화재</t>
+          <t>이수페타시스</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>33740.16</v>
+        <v>9296.65</v>
       </c>
       <c r="D135" t="n">
-        <v>1487.79</v>
+        <v>1521.39</v>
       </c>
       <c r="E135" t="n">
-        <v>1067.22</v>
+        <v>1578.55</v>
       </c>
       <c r="F135" t="n">
-        <v>128946.89</v>
+        <v>11878.47</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -4090,20 +4090,20 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CJ</t>
+          <t>한화투자증권</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2621.58</v>
+        <v>29855.48</v>
       </c>
       <c r="D136" t="n">
-        <v>1464.83</v>
+        <v>1509.05</v>
       </c>
       <c r="E136" t="n">
-        <v>1355.11</v>
+        <v>1000.49</v>
       </c>
       <c r="F136" t="n">
-        <v>33855.18</v>
+        <v>164528.46</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -4117,20 +4117,20 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>신영증권</t>
+          <t>현대엘리베이터</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>24057.52</v>
+        <v>16071</v>
       </c>
       <c r="D137" t="n">
-        <v>1455.17</v>
+        <v>1508.32</v>
       </c>
       <c r="E137" t="n">
-        <v>1181.51</v>
+        <v>3111.36</v>
       </c>
       <c r="F137" t="n">
-        <v>98188.64999999999</v>
+        <v>27628.05</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -4144,20 +4144,20 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>세방전지</t>
+          <t>대상</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>15820.33</v>
+        <v>35288.56</v>
       </c>
       <c r="D138" t="n">
-        <v>1424.97</v>
+        <v>1505.19</v>
       </c>
       <c r="E138" t="n">
-        <v>1494.72</v>
+        <v>-2855.56</v>
       </c>
       <c r="F138" t="n">
-        <v>17638.03</v>
+        <v>30613.98</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -4171,20 +4171,20 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>한솔케미칼</t>
+          <t>한국콜마</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>6831.82</v>
+        <v>11927.52</v>
       </c>
       <c r="D139" t="n">
-        <v>1399.96</v>
+        <v>1495.33</v>
       </c>
       <c r="E139" t="n">
-        <v>1387.79</v>
+        <v>1142.71</v>
       </c>
       <c r="F139" t="n">
-        <v>12663.1</v>
+        <v>15290.03</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -4198,20 +4198,20 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>한전KPS</t>
+          <t>CJ</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>15452.56</v>
+        <v>2621.58</v>
       </c>
       <c r="D140" t="n">
-        <v>1393.76</v>
+        <v>1464.83</v>
       </c>
       <c r="E140" t="n">
-        <v>1237.96</v>
+        <v>1355.11</v>
       </c>
       <c r="F140" t="n">
-        <v>16877.6</v>
+        <v>33855.18</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -4225,20 +4225,20 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>효성티앤씨</t>
+          <t>신영증권</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>43251.72</v>
+        <v>24057.52</v>
       </c>
       <c r="D141" t="n">
-        <v>1392.14</v>
+        <v>1455.17</v>
       </c>
       <c r="E141" t="n">
-        <v>1437.46</v>
+        <v>1181.51</v>
       </c>
       <c r="F141" t="n">
-        <v>22969.8</v>
+        <v>98188.64999999999</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -4252,20 +4252,20 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>세방전지</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>34084.92</v>
+        <v>16365.25</v>
       </c>
       <c r="D142" t="n">
-        <v>1373.86</v>
+        <v>1447.34</v>
       </c>
       <c r="E142" t="n">
-        <v>1210.02</v>
+        <v>1415.84</v>
       </c>
       <c r="F142" t="n">
-        <v>173152.31</v>
+        <v>18784.55</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -4279,20 +4279,20 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>한세실업</t>
+          <t>한솔케미칼</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>17190.24</v>
+        <v>6831.82</v>
       </c>
       <c r="D143" t="n">
-        <v>1355.28</v>
+        <v>1399.96</v>
       </c>
       <c r="E143" t="n">
-        <v>800.01</v>
+        <v>1387.79</v>
       </c>
       <c r="F143" t="n">
-        <v>11432.63</v>
+        <v>12663.1</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -4306,20 +4306,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>iM금융지주</t>
+          <t>한전KPS</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2404.29</v>
+        <v>15452.56</v>
       </c>
       <c r="D144" t="n">
-        <v>1354.23</v>
+        <v>1393.76</v>
       </c>
       <c r="E144" t="n">
-        <v>1359.64</v>
+        <v>1237.96</v>
       </c>
       <c r="F144" t="n">
-        <v>47399.91</v>
+        <v>16877.6</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -4333,20 +4333,20 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>롯데지주</t>
+          <t>효성티앤씨</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3391.18</v>
+        <v>43251.72</v>
       </c>
       <c r="D145" t="n">
-        <v>1341.88</v>
+        <v>1392.14</v>
       </c>
       <c r="E145" t="n">
-        <v>754.03</v>
+        <v>1437.46</v>
       </c>
       <c r="F145" t="n">
-        <v>90920.25999999999</v>
+        <v>22969.8</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -4360,20 +4360,20 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>농심</t>
+          <t>한국카본</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>27347.14</v>
+        <v>8663.74</v>
       </c>
       <c r="D146" t="n">
-        <v>1338.22</v>
+        <v>1382.12</v>
       </c>
       <c r="E146" t="n">
-        <v>1388.78</v>
+        <v>997.17</v>
       </c>
       <c r="F146" t="n">
-        <v>32321.21</v>
+        <v>10330.23</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -4387,20 +4387,20 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>KG스틸</t>
+          <t>대한해운</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>29263.88</v>
+        <v>6142.23</v>
       </c>
       <c r="D147" t="n">
-        <v>1335.13</v>
+        <v>1344.01</v>
       </c>
       <c r="E147" t="n">
-        <v>1194.31</v>
+        <v>1833.51</v>
       </c>
       <c r="F147" t="n">
-        <v>29746.49</v>
+        <v>20033.19</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -4414,20 +4414,20 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>케이뱅크</t>
+          <t>롯데지주</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>12285.01</v>
+        <v>3391.18</v>
       </c>
       <c r="D148" t="n">
-        <v>1329.67</v>
+        <v>1341.88</v>
       </c>
       <c r="E148" t="n">
-        <v>1280.53</v>
+        <v>754.03</v>
       </c>
       <c r="F148" t="n">
-        <v>311833.99</v>
+        <v>90920.25999999999</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -4441,20 +4441,20 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>농심</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>11141.23</v>
+        <v>27347.14</v>
       </c>
       <c r="D149" t="n">
-        <v>1327.01</v>
+        <v>1338.22</v>
       </c>
       <c r="E149" t="n">
-        <v>1305.88</v>
+        <v>1388.78</v>
       </c>
       <c r="F149" t="n">
-        <v>14128.13</v>
+        <v>32321.21</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -4468,20 +4468,20 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>경동나비엔</t>
+          <t>KG스틸</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>12635.45</v>
+        <v>29263.88</v>
       </c>
       <c r="D150" t="n">
-        <v>1317.96</v>
+        <v>1335.13</v>
       </c>
       <c r="E150" t="n">
-        <v>822.85</v>
+        <v>1194.31</v>
       </c>
       <c r="F150" t="n">
-        <v>10845.89</v>
+        <v>29746.49</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -4495,20 +4495,20 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>경동나비엔</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>13710.57</v>
+        <v>12635.45</v>
       </c>
       <c r="D151" t="n">
-        <v>1300.66</v>
+        <v>1317.96</v>
       </c>
       <c r="E151" t="n">
-        <v>1737.53</v>
+        <v>822.85</v>
       </c>
       <c r="F151" t="n">
-        <v>16956.95</v>
+        <v>10845.89</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -4522,20 +4522,20 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>한일시멘트</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>10110.96</v>
+        <v>13710.57</v>
       </c>
       <c r="D152" t="n">
-        <v>1257.39</v>
+        <v>1300.66</v>
       </c>
       <c r="E152" t="n">
-        <v>857.46</v>
+        <v>1737.53</v>
       </c>
       <c r="F152" t="n">
-        <v>30007.28</v>
+        <v>16956.95</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -4549,20 +4549,20 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>서연이화</t>
+          <t>한일시멘트</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>19254.2</v>
+        <v>10110.96</v>
       </c>
       <c r="D153" t="n">
-        <v>1233.56</v>
+        <v>1257.39</v>
       </c>
       <c r="E153" t="n">
-        <v>175.7</v>
+        <v>857.46</v>
       </c>
       <c r="F153" t="n">
-        <v>18152.93</v>
+        <v>30007.28</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -4576,20 +4576,20 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>영원무역홀딩스</t>
+          <t>서연이화</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1514.61</v>
+        <v>19254.2</v>
       </c>
       <c r="D154" t="n">
-        <v>1220.16</v>
+        <v>1233.56</v>
       </c>
       <c r="E154" t="n">
-        <v>1241.82</v>
+        <v>175.7</v>
       </c>
       <c r="F154" t="n">
-        <v>7242.69</v>
+        <v>18152.93</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -4603,20 +4603,20 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>HL홀딩스</t>
+          <t>영원무역홀딩스</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>9474.16</v>
+        <v>1535.79</v>
       </c>
       <c r="D155" t="n">
-        <v>1193.99</v>
+        <v>1230.82</v>
       </c>
       <c r="E155" t="n">
-        <v>373.36</v>
+        <v>1175.44</v>
       </c>
       <c r="F155" t="n">
-        <v>21787.92</v>
+        <v>7608.75</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -4630,20 +4630,20 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>미래에셋생명</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>46539.62</v>
+        <v>13348.3</v>
       </c>
       <c r="D156" t="n">
-        <v>1149.39</v>
+        <v>1170.85</v>
       </c>
       <c r="E156" t="n">
-        <v>1250.39</v>
+        <v>1126.09</v>
       </c>
       <c r="F156" t="n">
-        <v>324044.39</v>
+        <v>318642.88</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -4684,20 +4684,20 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>유한양행</t>
+          <t>KSS해운</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>21056.61</v>
+        <v>5613.49</v>
       </c>
       <c r="D158" t="n">
-        <v>1101.96</v>
+        <v>1103.06</v>
       </c>
       <c r="E158" t="n">
-        <v>2095.66</v>
+        <v>365.17</v>
       </c>
       <c r="F158" t="n">
-        <v>27138.37</v>
+        <v>19332.37</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -4711,20 +4711,20 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>SNT모티브</t>
+          <t>유한양행</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9987.389999999999</v>
+        <v>21056.61</v>
       </c>
       <c r="D159" t="n">
-        <v>1091.61</v>
+        <v>1101.96</v>
       </c>
       <c r="E159" t="n">
-        <v>760.4</v>
+        <v>2095.66</v>
       </c>
       <c r="F159" t="n">
-        <v>12681.8</v>
+        <v>27138.37</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -4738,20 +4738,20 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>쿠쿠홈시스</t>
+          <t>SNT모티브</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>8066.44</v>
+        <v>9987.389999999999</v>
       </c>
       <c r="D160" t="n">
-        <v>1085.42</v>
+        <v>1091.61</v>
       </c>
       <c r="E160" t="n">
-        <v>1187.4</v>
+        <v>760.4</v>
       </c>
       <c r="F160" t="n">
-        <v>10494.67</v>
+        <v>12681.8</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -4765,20 +4765,20 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>INVENI</t>
+          <t>쿠쿠홈시스</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1728.82</v>
+        <v>8066.44</v>
       </c>
       <c r="D161" t="n">
-        <v>1078.85</v>
+        <v>1085.42</v>
       </c>
       <c r="E161" t="n">
-        <v>857.29</v>
+        <v>1187.4</v>
       </c>
       <c r="F161" t="n">
-        <v>8289.09</v>
+        <v>10494.67</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -4792,20 +4792,20 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>DN오토모티브</t>
+          <t>INVENI</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>9862.799999999999</v>
+        <v>1728.82</v>
       </c>
       <c r="D162" t="n">
-        <v>1071.15</v>
+        <v>1078.85</v>
       </c>
       <c r="E162" t="n">
-        <v>689.6799999999999</v>
+        <v>857.29</v>
       </c>
       <c r="F162" t="n">
-        <v>19240.2</v>
+        <v>8289.09</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -4819,20 +4819,20 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>DN오토모티브</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>31182.23</v>
+        <v>9862.799999999999</v>
       </c>
       <c r="D163" t="n">
-        <v>1069.43</v>
+        <v>1071.15</v>
       </c>
       <c r="E163" t="n">
-        <v>762.59</v>
+        <v>689.6799999999999</v>
       </c>
       <c r="F163" t="n">
-        <v>32302.89</v>
+        <v>19240.2</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -4846,20 +4846,20 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>LX세미콘</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>16390.71</v>
+        <v>31182.23</v>
       </c>
       <c r="D164" t="n">
-        <v>1055.77</v>
+        <v>1069.43</v>
       </c>
       <c r="E164" t="n">
-        <v>824.99</v>
+        <v>762.59</v>
       </c>
       <c r="F164" t="n">
-        <v>13862.72</v>
+        <v>32302.89</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -4873,20 +4873,20 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>KSS해운</t>
+          <t>LX세미콘</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>5178.86</v>
+        <v>16390.71</v>
       </c>
       <c r="D165" t="n">
-        <v>1040.71</v>
+        <v>1055.77</v>
       </c>
       <c r="E165" t="n">
-        <v>573.85</v>
+        <v>824.99</v>
       </c>
       <c r="F165" t="n">
-        <v>18909.83</v>
+        <v>13862.72</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -4954,20 +4954,20 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>NHN</t>
+          <t>유안타증권</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3743.93</v>
+        <v>34119.73</v>
       </c>
       <c r="D168" t="n">
-        <v>1004.22</v>
+        <v>1006.31</v>
       </c>
       <c r="E168" t="n">
-        <v>218.5</v>
+        <v>853.5599999999999</v>
       </c>
       <c r="F168" t="n">
-        <v>18630.58</v>
+        <v>192903.24</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -5008,20 +5008,20 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>제일기획</t>
+          <t>달바글로벌</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>14156.23</v>
+        <v>5025.89</v>
       </c>
       <c r="D170" t="n">
-        <v>972</v>
+        <v>990.88</v>
       </c>
       <c r="E170" t="n">
-        <v>1059.79</v>
+        <v>767.21</v>
       </c>
       <c r="F170" t="n">
-        <v>12749.87</v>
+        <v>2535.24</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -5035,20 +5035,20 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>JW중외제약</t>
+          <t>제일기획</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>7671.5</v>
+        <v>14156.23</v>
       </c>
       <c r="D171" t="n">
-        <v>966.3</v>
+        <v>972</v>
       </c>
       <c r="E171" t="n">
-        <v>613.1</v>
+        <v>1059.79</v>
       </c>
       <c r="F171" t="n">
-        <v>5959.35</v>
+        <v>12749.87</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -5062,20 +5062,20 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>JW중외제약</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>11406.2</v>
+        <v>7671.5</v>
       </c>
       <c r="D172" t="n">
-        <v>958.21</v>
+        <v>966.3</v>
       </c>
       <c r="E172" t="n">
-        <v>986.53</v>
+        <v>613.1</v>
       </c>
       <c r="F172" t="n">
-        <v>19353.88</v>
+        <v>5959.35</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -5089,20 +5089,20 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SK케미칼</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>14403.81</v>
+        <v>11406.2</v>
       </c>
       <c r="D173" t="n">
-        <v>957.13</v>
+        <v>958.21</v>
       </c>
       <c r="E173" t="n">
-        <v>689.76</v>
+        <v>986.53</v>
       </c>
       <c r="F173" t="n">
-        <v>23232.52</v>
+        <v>19353.88</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -5116,20 +5116,20 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>SNT에너지</t>
+          <t>SK케미칼</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>4991.46</v>
+        <v>14403.81</v>
       </c>
       <c r="D174" t="n">
-        <v>955.37</v>
+        <v>957.13</v>
       </c>
       <c r="E174" t="n">
-        <v>741.41</v>
+        <v>689.76</v>
       </c>
       <c r="F174" t="n">
-        <v>5261.4</v>
+        <v>23232.52</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -5143,20 +5143,20 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>SNT에너지</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>21500.89</v>
+        <v>4991.46</v>
       </c>
       <c r="D175" t="n">
-        <v>910.37</v>
+        <v>955.37</v>
       </c>
       <c r="E175" t="n">
-        <v>510.71</v>
+        <v>741.41</v>
       </c>
       <c r="F175" t="n">
-        <v>24212.92</v>
+        <v>5261.4</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -5170,20 +5170,20 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>NICE평가정보</t>
+          <t>한세실업</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>4759.14</v>
+        <v>18279.33</v>
       </c>
       <c r="D176" t="n">
-        <v>906.97</v>
+        <v>939.11</v>
       </c>
       <c r="E176" t="n">
-        <v>689.2</v>
+        <v>511.95</v>
       </c>
       <c r="F176" t="n">
-        <v>5568.22</v>
+        <v>11775.99</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -5197,20 +5197,20 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>유안타증권</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>26720.77</v>
+        <v>21500.89</v>
       </c>
       <c r="D177" t="n">
-        <v>906.36</v>
+        <v>910.37</v>
       </c>
       <c r="E177" t="n">
-        <v>902.75</v>
+        <v>510.71</v>
       </c>
       <c r="F177" t="n">
-        <v>161325.78</v>
+        <v>24212.92</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -5224,20 +5224,20 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>명인제약</t>
+          <t>NICE평가정보</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2695.86</v>
+        <v>4759.14</v>
       </c>
       <c r="D178" t="n">
-        <v>900.58</v>
+        <v>906.97</v>
       </c>
       <c r="E178" t="n">
-        <v>661.52</v>
+        <v>689.2</v>
       </c>
       <c r="F178" t="n">
-        <v>5729.23</v>
+        <v>5568.22</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -5251,20 +5251,20 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>오뚜기</t>
+          <t>명인제약</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>29886.55</v>
+        <v>2873.64</v>
       </c>
       <c r="D179" t="n">
-        <v>893.8099999999999</v>
+        <v>899.21</v>
       </c>
       <c r="E179" t="n">
-        <v>617.72</v>
+        <v>792.51</v>
       </c>
       <c r="F179" t="n">
-        <v>25944.56</v>
+        <v>8315.370000000001</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -5278,20 +5278,20 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>오뚜기</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>178001.26</v>
+        <v>29886.55</v>
       </c>
       <c r="D180" t="n">
-        <v>892.35</v>
+        <v>893.8099999999999</v>
       </c>
       <c r="E180" t="n">
-        <v>-409.17</v>
+        <v>617.72</v>
       </c>
       <c r="F180" t="n">
-        <v>314554.55</v>
+        <v>25944.56</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -5305,20 +5305,20 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>롯데웰푸드</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>32828.57</v>
+        <v>178001.26</v>
       </c>
       <c r="D181" t="n">
-        <v>842.35</v>
+        <v>892.35</v>
       </c>
       <c r="E181" t="n">
-        <v>661.52</v>
+        <v>-409.17</v>
       </c>
       <c r="F181" t="n">
-        <v>41168.64</v>
+        <v>314554.55</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -5332,20 +5332,20 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>SNT다이내믹스</t>
+          <t>롯데웰푸드</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>6051.36</v>
+        <v>32828.57</v>
       </c>
       <c r="D182" t="n">
-        <v>833.74</v>
+        <v>842.35</v>
       </c>
       <c r="E182" t="n">
-        <v>598.92</v>
+        <v>661.52</v>
       </c>
       <c r="F182" t="n">
-        <v>11983.81</v>
+        <v>41168.64</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -5359,20 +5359,20 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>한국단자</t>
+          <t>SNT다이내믹스</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>11706.86</v>
+        <v>6051.36</v>
       </c>
       <c r="D183" t="n">
-        <v>825.5700000000001</v>
+        <v>833.74</v>
       </c>
       <c r="E183" t="n">
-        <v>670.95</v>
+        <v>598.92</v>
       </c>
       <c r="F183" t="n">
-        <v>12653.33</v>
+        <v>11983.81</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -5386,20 +5386,20 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>동원시스템즈</t>
+          <t>한국단자</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>12301.44</v>
+        <v>11706.86</v>
       </c>
       <c r="D184" t="n">
-        <v>811.66</v>
+        <v>825.5700000000001</v>
       </c>
       <c r="E184" t="n">
-        <v>865.14</v>
+        <v>670.95</v>
       </c>
       <c r="F184" t="n">
-        <v>14835.59</v>
+        <v>12653.33</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -5440,20 +5440,20 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>이수페타시스</t>
+          <t>NHN</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>7187.29</v>
+        <v>3748.22</v>
       </c>
       <c r="D186" t="n">
-        <v>784.8</v>
+        <v>795.23</v>
       </c>
       <c r="E186" t="n">
-        <v>652.48</v>
+        <v>3.32</v>
       </c>
       <c r="F186" t="n">
-        <v>6871.52</v>
+        <v>18307.59</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -5467,20 +5467,20 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>현대홈쇼핑</t>
+          <t>HL홀딩스</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>10898.89</v>
+        <v>8728.23</v>
       </c>
       <c r="D187" t="n">
-        <v>773.33</v>
+        <v>777.73</v>
       </c>
       <c r="E187" t="n">
-        <v>946.41</v>
+        <v>127.95</v>
       </c>
       <c r="F187" t="n">
-        <v>18981.43</v>
+        <v>21244.56</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -5494,20 +5494,20 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>녹십자</t>
+          <t>현대홈쇼핑</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>14603.54</v>
+        <v>10898.89</v>
       </c>
       <c r="D188" t="n">
-        <v>765.24</v>
+        <v>773.33</v>
       </c>
       <c r="E188" t="n">
-        <v>485.4</v>
+        <v>946.41</v>
       </c>
       <c r="F188" t="n">
-        <v>23917.58</v>
+        <v>18981.43</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -5521,20 +5521,20 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>케이카</t>
+          <t>녹십자</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>24388.39</v>
+        <v>14603.54</v>
       </c>
       <c r="D189" t="n">
-        <v>759.74</v>
+        <v>765.24</v>
       </c>
       <c r="E189" t="n">
-        <v>508.86</v>
+        <v>485.4</v>
       </c>
       <c r="F189" t="n">
-        <v>5345.7</v>
+        <v>23917.58</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -5548,20 +5548,20 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>AJ네트웍스</t>
+          <t>케이카</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>6982.77</v>
+        <v>24388.39</v>
       </c>
       <c r="D190" t="n">
-        <v>750.92</v>
+        <v>759.74</v>
       </c>
       <c r="E190" t="n">
-        <v>286.31</v>
+        <v>508.86</v>
       </c>
       <c r="F190" t="n">
-        <v>17031.29</v>
+        <v>5345.7</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -5575,20 +5575,20 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>롯데정밀화학</t>
+          <t>한양증권</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>17503.45</v>
+        <v>9090.219999999999</v>
       </c>
       <c r="D191" t="n">
-        <v>745.12</v>
+        <v>753.11</v>
       </c>
       <c r="E191" t="n">
-        <v>1030.29</v>
+        <v>565.71</v>
       </c>
       <c r="F191" t="n">
-        <v>25389.86</v>
+        <v>18337.01</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -5602,20 +5602,20 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>현대코퍼레이션</t>
+          <t>AJ네트웍스</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>52558.5</v>
+        <v>6982.77</v>
       </c>
       <c r="D192" t="n">
-        <v>732.89</v>
+        <v>750.92</v>
       </c>
       <c r="E192" t="n">
-        <v>864.4299999999999</v>
+        <v>286.31</v>
       </c>
       <c r="F192" t="n">
-        <v>16802.64</v>
+        <v>17031.29</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -5629,20 +5629,20 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>빙그레</t>
+          <t>롯데정밀화학</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>13124.34</v>
+        <v>17503.45</v>
       </c>
       <c r="D193" t="n">
-        <v>730.79</v>
+        <v>745.12</v>
       </c>
       <c r="E193" t="n">
-        <v>519.89</v>
+        <v>1030.29</v>
       </c>
       <c r="F193" t="n">
-        <v>10157.36</v>
+        <v>25389.86</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -5656,20 +5656,20 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>SNT홀딩스</t>
+          <t>현대코퍼레이션</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>765.9</v>
+        <v>52558.5</v>
       </c>
       <c r="D194" t="n">
-        <v>727.72</v>
+        <v>732.89</v>
       </c>
       <c r="E194" t="n">
-        <v>1374.78</v>
+        <v>864.4299999999999</v>
       </c>
       <c r="F194" t="n">
-        <v>6049.49</v>
+        <v>16802.64</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -5683,20 +5683,20 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>덴티움</t>
+          <t>빙그레</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>3207.23</v>
+        <v>13124.34</v>
       </c>
       <c r="D195" t="n">
-        <v>706.26</v>
+        <v>730.79</v>
       </c>
       <c r="E195" t="n">
-        <v>267.33</v>
+        <v>519.89</v>
       </c>
       <c r="F195" t="n">
-        <v>7373.13</v>
+        <v>10157.36</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -5710,20 +5710,20 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>세아베스틸지주</t>
+          <t>SNT홀딩스</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>883.78</v>
+        <v>765.9</v>
       </c>
       <c r="D196" t="n">
-        <v>702.03</v>
+        <v>727.72</v>
       </c>
       <c r="E196" t="n">
-        <v>643.42</v>
+        <v>1374.78</v>
       </c>
       <c r="F196" t="n">
-        <v>18317.64</v>
+        <v>6049.49</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -5737,20 +5737,20 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>LX홀딩스</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1041.2</v>
+        <v>16617.81</v>
       </c>
       <c r="D197" t="n">
-        <v>701.53</v>
+        <v>716.2</v>
       </c>
       <c r="E197" t="n">
-        <v>757.67</v>
+        <v>534.89</v>
       </c>
       <c r="F197" t="n">
-        <v>14084.78</v>
+        <v>107668.53</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -5764,20 +5764,20 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>HD현대마린엔진</t>
+          <t>세아베스틸지주</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3798.48</v>
+        <v>883.78</v>
       </c>
       <c r="D198" t="n">
-        <v>684.52</v>
+        <v>702.03</v>
       </c>
       <c r="E198" t="n">
-        <v>1573.79</v>
+        <v>643.42</v>
       </c>
       <c r="F198" t="n">
-        <v>7833.44</v>
+        <v>18317.64</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -5791,20 +5791,20 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>TKG휴켐스</t>
+          <t>LX홀딩스</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>10822.36</v>
+        <v>1041.2</v>
       </c>
       <c r="D199" t="n">
-        <v>674.71</v>
+        <v>701.53</v>
       </c>
       <c r="E199" t="n">
-        <v>611.71</v>
+        <v>757.67</v>
       </c>
       <c r="F199" t="n">
-        <v>10694.35</v>
+        <v>14084.78</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -5818,20 +5818,20 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>보령</t>
+          <t>현대차증권</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>9678.110000000001</v>
+        <v>17951.75</v>
       </c>
       <c r="D200" t="n">
-        <v>673.4</v>
+        <v>687.1799999999999</v>
       </c>
       <c r="E200" t="n">
-        <v>699.6799999999999</v>
+        <v>541.9</v>
       </c>
       <c r="F200" t="n">
-        <v>13738</v>
+        <v>116761.87</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -5845,20 +5845,20 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>HL D&amp;I</t>
+          <t>HD현대마린엔진</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>16451.9</v>
+        <v>3798.48</v>
       </c>
       <c r="D201" t="n">
-        <v>672.03</v>
+        <v>684.52</v>
       </c>
       <c r="E201" t="n">
-        <v>244.39</v>
+        <v>1573.79</v>
       </c>
       <c r="F201" t="n">
-        <v>16806.03</v>
+        <v>7833.44</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-04-01 02:27</t>
+          <t>2026-07-01 03:36</t>
         </is>
       </c>
     </row>

</xml_diff>